<commit_message>
Validation workbook: add Sheet 6 (full-text reports without a local PDF, 90 records, risk-sorted) so the author can obtain and re-decide every full-text call that could not be checked against the full text; the 9 'not retrieved' exclusions are the main missed-study risk
</commit_message>
<xml_diff>
--- a/meta_agents/search_v2/outputs/Author_Validation_Workbook.xlsx
+++ b/meta_agents/search_v2/outputs/Author_Validation_Workbook.xlsx
@@ -13,12 +13,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2_TA_Excluded_Sample" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_Extraction_Verification" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4_RoB_Review" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6_FullText_ToObtain" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'1_FullText_Inclusion'!$A$1:$I$244</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'2_TA_Excluded_Sample'!$A$1:$E$152</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'3_Extraction_Verification'!$A$1:$M$149</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'4_RoB_Review'!$A$1:$Q$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'6_FullText_ToObtain'!$A$1:$I$92</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -293,6 +295,21 @@
     <comment ref="J1" authorId="0" shapeId="0">
       <text>
         <t>Where in the source the value came from — go here to confirm the extracted numbers.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>validation</author>
+  </authors>
+  <commentList>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>HIGH: a 'not retrieved' exclusion (a study we could not obtain, so eligibility is unconfirmed — the main risk of a missed study) or a quantitative estimate extracted without the main PDF. Obtain these first.</t>
       </text>
     </comment>
   </commentList>
@@ -588,7 +605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -687,22 +704,43 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
+          <t>Sheet 6 — Full-text to obtain (90 reports with no local PDF): obtain each and confirm/override the</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        include/exclude decision (cols G–H). HIGH-risk rows first — these are studies we could not</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        retrieve, the main place an eligible study could have been missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
           <t>Sheet 5 — Summary: agreement rates, computed automatically. Nothing to fill here.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Row 2 of each sheet is a grey EXAMPLE row showing the expected format — delete it before finalizing.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>Yellow = you fill.  White = AI reference (do not edit).  Dropdowns are provided where applicable.</t>
         </is>
@@ -719,7 +757,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -938,8 +976,59 @@
         <v/>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Full-text reports to obtain (Sheet 6)</t>
+        </is>
+      </c>
+    </row>
     <row r="24">
-      <c r="A24" s="9" t="inlineStr">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Reports without local PDF</t>
+        </is>
+      </c>
+      <c r="B24" s="7">
+        <f>COUNTA('6_FullText_ToObtain'!A3:A400)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  HIGH-risk (obtain first)</t>
+        </is>
+      </c>
+      <c r="B25" s="7">
+        <f>COUNTIF('6_FullText_ToObtain'!F3:F400,"HIGH*")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Author obtained</t>
+        </is>
+      </c>
+      <c r="B26" s="7">
+        <f>COUNTA('6_FullText_ToObtain'!G3:G400)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Obtained rate</t>
+        </is>
+      </c>
+      <c r="B27" s="8">
+        <f>IFERROR(B26/B24,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
         <is>
           <t>Rates populate automatically as you fill the yellow columns in each sheet.</t>
         </is>
@@ -14490,12 +14579,12 @@
       </c>
       <c r="G41" s="13" t="inlineStr">
         <is>
-          <t>143</t>
+          <t>140.4 [137.6, 143.2]</t>
         </is>
       </c>
       <c r="H41" s="13" t="inlineStr">
         <is>
-          <t>0.755 [0.677, 0.842]</t>
+          <t>0.769 [0.688, 0.860]</t>
         </is>
       </c>
       <c r="I41" s="14" t="inlineStr">
@@ -14505,7 +14594,7 @@
       </c>
       <c r="J41" s="14" t="inlineStr">
         <is>
-          <t>Table 4 (female breast)</t>
+          <t>Table 4 (origin female-breast rates); Table 2 (NHW-FL reference)</t>
         </is>
       </c>
       <c r="K41" s="15" t="inlineStr"/>
@@ -14545,12 +14634,12 @@
       </c>
       <c r="G42" s="13" t="inlineStr">
         <is>
-          <t>143</t>
+          <t>140.4 [137.6, 143.2]</t>
         </is>
       </c>
       <c r="H42" s="13" t="inlineStr">
         <is>
-          <t>0.503 [0.376, 0.673]</t>
+          <t>0.512 [0.382, 0.686]</t>
         </is>
       </c>
       <c r="I42" s="14" t="inlineStr">
@@ -14560,7 +14649,7 @@
       </c>
       <c r="J42" s="14" t="inlineStr">
         <is>
-          <t>Table 4 (female breast)</t>
+          <t>Table 4 (origin female-breast rates); Table 2 (NHW-FL reference)</t>
         </is>
       </c>
       <c r="K42" s="15" t="inlineStr"/>
@@ -14600,12 +14689,12 @@
       </c>
       <c r="G43" s="13" t="inlineStr">
         <is>
-          <t>143</t>
+          <t>140.4 [137.6, 143.2]</t>
         </is>
       </c>
       <c r="H43" s="13" t="inlineStr">
         <is>
-          <t>0.817 [0.726, 0.920]</t>
+          <t>0.833 [0.738, 0.939]</t>
         </is>
       </c>
       <c r="I43" s="14" t="inlineStr">
@@ -14615,7 +14704,7 @@
       </c>
       <c r="J43" s="14" t="inlineStr">
         <is>
-          <t>Table 4 (female breast)</t>
+          <t>Table 4 (origin female-breast rates); Table 2 (NHW-FL reference)</t>
         </is>
       </c>
       <c r="K43" s="15" t="inlineStr"/>
@@ -14655,12 +14744,12 @@
       </c>
       <c r="G44" s="13" t="inlineStr">
         <is>
-          <t>143</t>
+          <t>140.4 [137.6, 143.2]</t>
         </is>
       </c>
       <c r="H44" s="13" t="inlineStr">
         <is>
-          <t>0.684 [0.619, 0.756]</t>
+          <t>0.697 [0.629, 0.771]</t>
         </is>
       </c>
       <c r="I44" s="14" t="inlineStr">
@@ -14670,7 +14759,7 @@
       </c>
       <c r="J44" s="14" t="inlineStr">
         <is>
-          <t>Table 4 (female breast)</t>
+          <t>Table 4 (origin female-breast rates); Table 2 (NHW-FL reference)</t>
         </is>
       </c>
       <c r="K44" s="15" t="inlineStr"/>
@@ -23571,4 +23660,3215 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I92"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>record_id</t>
+        </is>
+      </c>
+      <c r="B1" s="10" t="inlineStr">
+        <is>
+          <t>Current decision (AI)</t>
+        </is>
+      </c>
+      <c r="C1" s="10" t="inlineStr">
+        <is>
+          <t>Citation / title</t>
+        </is>
+      </c>
+      <c r="D1" s="10" t="inlineStr">
+        <is>
+          <t>PMID</t>
+        </is>
+      </c>
+      <c r="E1" s="10" t="inlineStr">
+        <is>
+          <t>DOI</t>
+        </is>
+      </c>
+      <c r="F1" s="10" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+      <c r="G1" s="10" t="inlineStr">
+        <is>
+          <t>AUTHOR obtained full text? (Yes/No)</t>
+        </is>
+      </c>
+      <c r="H1" s="10" t="inlineStr">
+        <is>
+          <t>AUTHOR final decision (Include/Exclude)</t>
+        </is>
+      </c>
+      <c r="I1" s="10" t="inlineStr">
+        <is>
+          <t>AUTHOR note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>e.g. 2038</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Full text unavailable)</t>
+        </is>
+      </c>
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>Incidence trends in TNBC...</t>
+        </is>
+      </c>
+      <c r="D2" s="11" t="inlineStr"/>
+      <c r="E2" s="11" t="inlineStr"/>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>HIGH — not retrieved (possible missed study)</t>
+        </is>
+      </c>
+      <c r="G2" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H2" s="11" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="I2" s="12" t="inlineStr">
+        <is>
+          <t>overlaps Sung 2023</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>155</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (quant-extracted)</t>
+        </is>
+      </c>
+      <c r="C3" s="14" t="inlineStr">
+        <is>
+          <t>State Variation in Racial and Ethnic Disparities in Incidence of Triple-Negative Breast Cancer among US Women (2023)</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>36862439</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>10.1001/jamaoncol.2022.7835</t>
+        </is>
+      </c>
+      <c r="F3" s="14" t="inlineStr">
+        <is>
+          <t>HIGH — extracted without main PDF</t>
+        </is>
+      </c>
+      <c r="G3" s="15" t="inlineStr"/>
+      <c r="H3" s="15" t="inlineStr"/>
+      <c r="I3" s="16" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>286</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (quant-extracted)</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>Variation in breast cancer subtype incidence and distribution by race/ethnicity in the United States from 2010 to 2015 (2020)</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>33074325</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>10.1001/jamanetworkopen.2020.20303</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>HIGH — extracted without main PDF</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="inlineStr"/>
+      <c r="H4" s="15" t="inlineStr"/>
+      <c r="I4" s="16" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>157</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Full text unavailable)</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>Breast cancer trends among black and white women in the United States (2005)</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>16258086</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>10.1200/jco.2004.01.0421</t>
+        </is>
+      </c>
+      <c r="F5" s="14" t="inlineStr">
+        <is>
+          <t>HIGH — not retrieved (possible missed study)</t>
+        </is>
+      </c>
+      <c r="G5" s="15" t="inlineStr"/>
+      <c r="H5" s="15" t="inlineStr"/>
+      <c r="I5" s="16" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>253</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Full text unavailable)</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>Breast cancer patterns and lifetime risk of developing breast cancer among Puerto Rican females. (2000)</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>10761199</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="inlineStr"/>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>HIGH — not retrieved (possible missed study)</t>
+        </is>
+      </c>
+      <c r="G6" s="15" t="inlineStr"/>
+      <c r="H6" s="15" t="inlineStr"/>
+      <c r="I6" s="16" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>415</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Full text unavailable)</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>Women's cancers among Alaska Natives 1969-2003. (2006)</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>17929614</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr"/>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>HIGH — not retrieved (possible missed study)</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="inlineStr"/>
+      <c r="H7" s="15" t="inlineStr"/>
+      <c r="I7" s="16" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>424</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Full text unavailable)</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>Breast cancer in a multiethnic cohort in Hawaii and Los Angeles: Risk factor-adjusted incidence in Japanese equals and in Hawaiians exceeds that in whites (2002)</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>12223421</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr"/>
+      <c r="F8" s="14" t="inlineStr">
+        <is>
+          <t>HIGH — not retrieved (possible missed study)</t>
+        </is>
+      </c>
+      <c r="G8" s="15" t="inlineStr"/>
+      <c r="H8" s="15" t="inlineStr"/>
+      <c r="I8" s="16" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>428</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Full text unavailable)</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>Women's cancers among Alaska Natives: [corrected] 1969-2003. (2007)</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>18323374</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr"/>
+      <c r="F9" s="14" t="inlineStr">
+        <is>
+          <t>HIGH — not retrieved (possible missed study)</t>
+        </is>
+      </c>
+      <c r="G9" s="15" t="inlineStr"/>
+      <c r="H9" s="15" t="inlineStr"/>
+      <c r="I9" s="16" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>476</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Full text unavailable)</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>Rural–urban disparities in breast cancer incidence among US women aged 20–49: trends by race/ethnicity, stage, poverty, and state from 2000–2019 (2026)</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>41665696</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>10.1007/s10552-026-02134-3</t>
+        </is>
+      </c>
+      <c r="F10" s="14" t="inlineStr">
+        <is>
+          <t>HIGH — not retrieved (possible missed study)</t>
+        </is>
+      </c>
+      <c r="G10" s="15" t="inlineStr"/>
+      <c r="H10" s="15" t="inlineStr"/>
+      <c r="I10" s="16" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>2038</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Full text unavailable)</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="inlineStr">
+        <is>
+          <t>Incidence trends in triple-negative breast cancer among women in the United States from 2010 to 2019 by race/ethnicity, age and tumor stage (2023)</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr"/>
+      <c r="E11" s="13" t="inlineStr"/>
+      <c r="F11" s="14" t="inlineStr">
+        <is>
+          <t>HIGH — not retrieved (possible missed study)</t>
+        </is>
+      </c>
+      <c r="G11" s="15" t="inlineStr"/>
+      <c r="H11" s="15" t="inlineStr"/>
+      <c r="I11" s="16" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>3116</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Full text unavailable)</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>Time trends and racial differences in female breast cancer incidence in Pennsylvania, 1985-2004 (2011)</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="inlineStr"/>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>10.1089/jwh.2010.2082</t>
+        </is>
+      </c>
+      <c r="F12" s="14" t="inlineStr">
+        <is>
+          <t>HIGH — not retrieved (possible missed study)</t>
+        </is>
+      </c>
+      <c r="G12" s="15" t="inlineStr"/>
+      <c r="H12" s="15" t="inlineStr"/>
+      <c r="I12" s="16" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>3268</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Full text unavailable)</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Improving cancer incidence estimates for American Indians in Wisconsin (2007)</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>17844709</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr"/>
+      <c r="F13" s="14" t="inlineStr">
+        <is>
+          <t>HIGH — not retrieved (possible missed study)</t>
+        </is>
+      </c>
+      <c r="G13" s="15" t="inlineStr"/>
+      <c r="H13" s="15" t="inlineStr"/>
+      <c r="I13" s="16" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>209</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (quant-eligible)</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>Racial and regional disparities of triple negative breast cancer incidence rates in the United States: An analysis of 2011-2019 NPCR and SEER incidence data (2022)</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>36530732</t>
+        </is>
+      </c>
+      <c r="E14" s="13" t="inlineStr">
+        <is>
+          <t>10.3389/fpubh.2022.1058722</t>
+        </is>
+      </c>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>MED — eligible, not extracted</t>
+        </is>
+      </c>
+      <c r="G14" s="15" t="inlineStr"/>
+      <c r="H14" s="15" t="inlineStr"/>
+      <c r="I14" s="16" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>419</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (quant-eligible)</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="inlineStr">
+        <is>
+          <t>Higher population-based incidence rates of triple-negative breast cancer among young African-American women (2011)</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>21656753</t>
+        </is>
+      </c>
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>10.1002/cncr.25862</t>
+        </is>
+      </c>
+      <c r="F15" s="14" t="inlineStr">
+        <is>
+          <t>MED — eligible, not extracted</t>
+        </is>
+      </c>
+      <c r="G15" s="15" t="inlineStr"/>
+      <c r="H15" s="15" t="inlineStr"/>
+      <c r="I15" s="16" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>2137</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (quant-eligible)</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="inlineStr">
+        <is>
+          <t>Cancer disparities among non-Hispanic urban American Indian and Alaska Native populations in the United States, 1999-2017 (2022)</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>35119703</t>
+        </is>
+      </c>
+      <c r="E16" s="13" t="inlineStr">
+        <is>
+          <t>10.1002/cncr.34122</t>
+        </is>
+      </c>
+      <c r="F16" s="14" t="inlineStr">
+        <is>
+          <t>MED — eligible, not extracted</t>
+        </is>
+      </c>
+      <c r="G16" s="15" t="inlineStr"/>
+      <c r="H16" s="15" t="inlineStr"/>
+      <c r="I16" s="16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>4027</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (quant-eligible)</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>Cancer incidence among Asian American populations in the United States, 2009-2011 (2016)</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>26661680</t>
+        </is>
+      </c>
+      <c r="E17" s="13" t="inlineStr">
+        <is>
+          <t>10.1002/ijc.29958</t>
+        </is>
+      </c>
+      <c r="F17" s="14" t="inlineStr">
+        <is>
+          <t>MED — eligible, not extracted</t>
+        </is>
+      </c>
+      <c r="G17" s="15" t="inlineStr"/>
+      <c r="H17" s="15" t="inlineStr"/>
+      <c r="I17" s="16" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Did not report the outcome of interest)</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>Stage IV Breast Cancer Incidence and Survival, 2010-202 (2026)</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>42118535</t>
+        </is>
+      </c>
+      <c r="E18" s="13" t="inlineStr">
+        <is>
+          <t>10.1001/jamanetworkopen.2026.12042</t>
+        </is>
+      </c>
+      <c r="F18" s="14" t="inlineStr">
+        <is>
+          <t>MED — excluded without full text</t>
+        </is>
+      </c>
+      <c r="G18" s="15" t="inlineStr"/>
+      <c r="H18" s="15" t="inlineStr"/>
+      <c r="I18" s="16" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>251</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Did not report the outcome of interest)</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>Triple-negative breast cancer incidence in the United States: ecological correlations with area-level sociodemographics, healthcare, and health behaviors (2021)</t>
+        </is>
+      </c>
+      <c r="D19" s="13" t="inlineStr">
+        <is>
+          <t>32671723</t>
+        </is>
+      </c>
+      <c r="E19" s="13" t="inlineStr">
+        <is>
+          <t>10.1007/s12282-020-01132-w</t>
+        </is>
+      </c>
+      <c r="F19" s="14" t="inlineStr">
+        <is>
+          <t>MED — excluded without full text</t>
+        </is>
+      </c>
+      <c r="G19" s="15" t="inlineStr"/>
+      <c r="H19" s="15" t="inlineStr"/>
+      <c r="I19" s="16" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>321</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Did not report the outcome of interest)</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="inlineStr">
+        <is>
+          <t>Risks of developing breast and colorectal cancer in association with incomes and geographic locations in Texas: A retrospective cohort study (2016)</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="inlineStr">
+        <is>
+          <t>27118258</t>
+        </is>
+      </c>
+      <c r="E20" s="13" t="inlineStr">
+        <is>
+          <t>10.1186/s12885-016-2324-z</t>
+        </is>
+      </c>
+      <c r="F20" s="14" t="inlineStr">
+        <is>
+          <t>MED — excluded without full text</t>
+        </is>
+      </c>
+      <c r="G20" s="15" t="inlineStr"/>
+      <c r="H20" s="15" t="inlineStr"/>
+      <c r="I20" s="16" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C21" s="14" t="inlineStr">
+        <is>
+          <t>Breast Cancer Incidence Trends in Older US Women by Race, Ethnicity, Geography, and Stage (2025)</t>
+        </is>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
+        <is>
+          <t>40553473</t>
+        </is>
+      </c>
+      <c r="E21" s="13" t="inlineStr">
+        <is>
+          <t>10.1001/jamanetworkopen.2025.16947</t>
+        </is>
+      </c>
+      <c r="F21" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G21" s="15" t="inlineStr"/>
+      <c r="H21" s="15" t="inlineStr"/>
+      <c r="I21" s="16" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C22" s="14" t="inlineStr">
+        <is>
+          <t>Invasive cancer incidence - United States, 2010. (2014)</t>
+        </is>
+      </c>
+      <c r="D22" s="13" t="inlineStr">
+        <is>
+          <t>24670926</t>
+        </is>
+      </c>
+      <c r="E22" s="13" t="inlineStr"/>
+      <c r="F22" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G22" s="15" t="inlineStr"/>
+      <c r="H22" s="15" t="inlineStr"/>
+      <c r="I22" s="16" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="inlineStr">
+        <is>
+          <t>Incidence Rate Trends of Breast Cancer Overall and by Molecular Subtype by Race and Ethnicity and Age (2025)</t>
+        </is>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
+        <is>
+          <t>39853979</t>
+        </is>
+      </c>
+      <c r="E23" s="13" t="inlineStr">
+        <is>
+          <t>10.1001/jamanetworkopen.2024.56142</t>
+        </is>
+      </c>
+      <c r="F23" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G23" s="15" t="inlineStr"/>
+      <c r="H23" s="15" t="inlineStr"/>
+      <c r="I23" s="16" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C24" s="14" t="inlineStr">
+        <is>
+          <t>Breast, Colorectal, and Prostate Cancer Incidence among Filipino Americans by Generational Status in the Multiethnic Cohort Study (2024)</t>
+        </is>
+      </c>
+      <c r="D24" s="13" t="inlineStr">
+        <is>
+          <t>39132985</t>
+        </is>
+      </c>
+      <c r="E24" s="13" t="inlineStr">
+        <is>
+          <t>10.1158/1055-9965.epi-24-0647</t>
+        </is>
+      </c>
+      <c r="F24" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G24" s="15" t="inlineStr"/>
+      <c r="H24" s="15" t="inlineStr"/>
+      <c r="I24" s="16" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>119</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C25" s="14" t="inlineStr">
+        <is>
+          <t>Disparities of cancer incidence in Michigan's American Indians: Spotlight on breast cancer (2014)</t>
+        </is>
+      </c>
+      <c r="D25" s="13" t="inlineStr">
+        <is>
+          <t>24676851</t>
+        </is>
+      </c>
+      <c r="E25" s="13" t="inlineStr">
+        <is>
+          <t>10.1002/cncr.28589</t>
+        </is>
+      </c>
+      <c r="F25" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G25" s="15" t="inlineStr"/>
+      <c r="H25" s="15" t="inlineStr"/>
+      <c r="I25" s="16" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>142</t>
+        </is>
+      </c>
+      <c r="B26" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C26" s="14" t="inlineStr">
+        <is>
+          <t>Are There Regional Differences in Triple Negative Breast Cancer among Non-Hispanic Black Women? (2021)</t>
+        </is>
+      </c>
+      <c r="D26" s="13" t="inlineStr">
+        <is>
+          <t>32778443</t>
+        </is>
+      </c>
+      <c r="E26" s="13" t="inlineStr">
+        <is>
+          <t>10.1016/j.jnma.2020.07.016</t>
+        </is>
+      </c>
+      <c r="F26" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G26" s="15" t="inlineStr"/>
+      <c r="H26" s="15" t="inlineStr"/>
+      <c r="I26" s="16" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>145</t>
+        </is>
+      </c>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="inlineStr">
+        <is>
+          <t>Persistence in breast cancer disparities between African Americans and whites in Wisconsin (2011)</t>
+        </is>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
+        <is>
+          <t>21473509</t>
+        </is>
+      </c>
+      <c r="E27" s="13" t="inlineStr"/>
+      <c r="F27" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G27" s="15" t="inlineStr"/>
+      <c r="H27" s="15" t="inlineStr"/>
+      <c r="I27" s="16" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>158</t>
+        </is>
+      </c>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="inlineStr">
+        <is>
+          <t>Trends in breast cancer incidence rates by race/ethnicity: Patterns by stage, socioeconomic position, and geography in the United States, 1999-2017 (2022)</t>
+        </is>
+      </c>
+      <c r="D28" s="13" t="inlineStr">
+        <is>
+          <t>34731501</t>
+        </is>
+      </c>
+      <c r="E28" s="13" t="inlineStr">
+        <is>
+          <t>10.1002/cncr.34008</t>
+        </is>
+      </c>
+      <c r="F28" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G28" s="15" t="inlineStr"/>
+      <c r="H28" s="15" t="inlineStr"/>
+      <c r="I28" s="16" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>210</t>
+        </is>
+      </c>
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C29" s="14" t="inlineStr">
+        <is>
+          <t>Breast cancer incidence trends in Asian women aged 20 or older as compared to other ethnic women in the United States from 2000 to 2018 by time period, age and tumor stage (2022)</t>
+        </is>
+      </c>
+      <c r="D29" s="13" t="inlineStr">
+        <is>
+          <t>34861613</t>
+        </is>
+      </c>
+      <c r="E29" s="13" t="inlineStr">
+        <is>
+          <t>10.1016/j.canep.2021.102076</t>
+        </is>
+      </c>
+      <c r="F29" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G29" s="15" t="inlineStr"/>
+      <c r="H29" s="15" t="inlineStr"/>
+      <c r="I29" s="16" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>226</t>
+        </is>
+      </c>
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C30" s="14" t="inlineStr">
+        <is>
+          <t>Home mortgage discrimination and incidence of triple-negative and Luminal A breast cancer among non-Hispanic Black and non-Hispanic White females in California, 2006–2015 (2022)</t>
+        </is>
+      </c>
+      <c r="D30" s="13" t="inlineStr">
+        <is>
+          <t>35113296</t>
+        </is>
+      </c>
+      <c r="E30" s="13" t="inlineStr">
+        <is>
+          <t>10.1007/s10552-022-01557-y</t>
+        </is>
+      </c>
+      <c r="F30" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G30" s="15" t="inlineStr"/>
+      <c r="H30" s="15" t="inlineStr"/>
+      <c r="I30" s="16" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>246</t>
+        </is>
+      </c>
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t>Does socioeconomic disparity in cancer incidence vary across racial/ethnic groups? (2010)</t>
+        </is>
+      </c>
+      <c r="D31" s="13" t="inlineStr">
+        <is>
+          <t>20567897</t>
+        </is>
+      </c>
+      <c r="E31" s="13" t="inlineStr">
+        <is>
+          <t>10.1007/s10552-010-9601-y</t>
+        </is>
+      </c>
+      <c r="F31" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G31" s="15" t="inlineStr"/>
+      <c r="H31" s="15" t="inlineStr"/>
+      <c r="I31" s="16" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>252</t>
+        </is>
+      </c>
+      <c r="B32" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C32" s="14" t="inlineStr">
+        <is>
+          <t>Forty-year trends in menopausal hormone therapy use and breast cancer incidence  among postmenopausal black and white women (2020)</t>
+        </is>
+      </c>
+      <c r="D32" s="13" t="inlineStr">
+        <is>
+          <t>32212335</t>
+        </is>
+      </c>
+      <c r="E32" s="13" t="inlineStr">
+        <is>
+          <t>10.1002/cncr.32846</t>
+        </is>
+      </c>
+      <c r="F32" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G32" s="15" t="inlineStr"/>
+      <c r="H32" s="15" t="inlineStr"/>
+      <c r="I32" s="16" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>259</t>
+        </is>
+      </c>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C33" s="14" t="inlineStr">
+        <is>
+          <t>What can we learn from the age- and race/ethnicity- specific rates of inflammatory breast carcinoma? (2011)</t>
+        </is>
+      </c>
+      <c r="D33" s="13" t="inlineStr">
+        <is>
+          <t>21850396</t>
+        </is>
+      </c>
+      <c r="E33" s="13" t="inlineStr">
+        <is>
+          <t>10.1007/s10549-011-1719-4</t>
+        </is>
+      </c>
+      <c r="F33" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G33" s="15" t="inlineStr"/>
+      <c r="H33" s="15" t="inlineStr"/>
+      <c r="I33" s="16" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="13" t="inlineStr">
+        <is>
+          <t>284</t>
+        </is>
+      </c>
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C34" s="14" t="inlineStr">
+        <is>
+          <t>Trends in Female Breast Cancer Incidence among Japanese, Korean, and US Populations: An Age-Period-Cohort Analysis (2026)</t>
+        </is>
+      </c>
+      <c r="D34" s="13" t="inlineStr">
+        <is>
+          <t>42065927</t>
+        </is>
+      </c>
+      <c r="E34" s="13" t="inlineStr">
+        <is>
+          <t>10.1158/1055-9965.epi-26-0101</t>
+        </is>
+      </c>
+      <c r="F34" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G34" s="15" t="inlineStr"/>
+      <c r="H34" s="15" t="inlineStr"/>
+      <c r="I34" s="16" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>310</t>
+        </is>
+      </c>
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C35" s="14" t="inlineStr">
+        <is>
+          <t>Recent breast cancer trends among Asian/Pacific Islander, Hispanic, and African-American women in the US: Changes by tumor subtype (2007)</t>
+        </is>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
+        <is>
+          <t>18162138</t>
+        </is>
+      </c>
+      <c r="E35" s="13" t="inlineStr">
+        <is>
+          <t>10.1186/bcr1839</t>
+        </is>
+      </c>
+      <c r="F35" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G35" s="15" t="inlineStr"/>
+      <c r="H35" s="15" t="inlineStr"/>
+      <c r="I35" s="16" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>316</t>
+        </is>
+      </c>
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C36" s="14" t="inlineStr">
+        <is>
+          <t>Early estimates of cancer incidence for 2015: Expanding to include estimates for white and black races (2018)</t>
+        </is>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
+        <is>
+          <t>29509274</t>
+        </is>
+      </c>
+      <c r="E36" s="13" t="inlineStr">
+        <is>
+          <t>10.1002/cncr.31315</t>
+        </is>
+      </c>
+      <c r="F36" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G36" s="15" t="inlineStr"/>
+      <c r="H36" s="15" t="inlineStr"/>
+      <c r="I36" s="16" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="13" t="inlineStr">
+        <is>
+          <t>369</t>
+        </is>
+      </c>
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C37" s="14" t="inlineStr">
+        <is>
+          <t>Differences in breast cancer incidence among young women aged 20–49 years by stage and tumor characteristics, age, race, and ethnicity, 2004–2013 (2018)</t>
+        </is>
+      </c>
+      <c r="D37" s="13" t="inlineStr">
+        <is>
+          <t>29445940</t>
+        </is>
+      </c>
+      <c r="E37" s="13" t="inlineStr">
+        <is>
+          <t>10.1007/s10549-018-4699-9</t>
+        </is>
+      </c>
+      <c r="F37" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G37" s="15" t="inlineStr"/>
+      <c r="H37" s="15" t="inlineStr"/>
+      <c r="I37" s="16" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="13" t="inlineStr">
+        <is>
+          <t>377</t>
+        </is>
+      </c>
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C38" s="14" t="inlineStr">
+        <is>
+          <t>Racial/ethnicity disparities in invasive breast cancer among younger and older  women: An analysis using multiple measures of population health (2016)</t>
+        </is>
+      </c>
+      <c r="D38" s="13" t="inlineStr">
+        <is>
+          <t>27792934</t>
+        </is>
+      </c>
+      <c r="E38" s="13" t="inlineStr">
+        <is>
+          <t>10.1016/j.canep.2016.10.013</t>
+        </is>
+      </c>
+      <c r="F38" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G38" s="15" t="inlineStr"/>
+      <c r="H38" s="15" t="inlineStr"/>
+      <c r="I38" s="16" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="13" t="inlineStr">
+        <is>
+          <t>402</t>
+        </is>
+      </c>
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C39" s="14" t="inlineStr">
+        <is>
+          <t>Disparities in Breast Cancer Incidence, Mortality, and Quality of Care among African American and European American Women in South Carolina (2016)</t>
+        </is>
+      </c>
+      <c r="D39" s="13" t="inlineStr">
+        <is>
+          <t>26741869</t>
+        </is>
+      </c>
+      <c r="E39" s="13" t="inlineStr">
+        <is>
+          <t>10.14423/smj.0000000000000396</t>
+        </is>
+      </c>
+      <c r="F39" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G39" s="15" t="inlineStr"/>
+      <c r="H39" s="15" t="inlineStr"/>
+      <c r="I39" s="16" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="13" t="inlineStr">
+        <is>
+          <t>426</t>
+        </is>
+      </c>
+      <c r="B40" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C40" s="14" t="inlineStr">
+        <is>
+          <t>Trends in Incidence of Invasive Lobular Carcinoma of the Breast by Race: Patterns by Age, Cancer Stage, and Socioeconomic Factors in the United States, 1992-2019 (2025)</t>
+        </is>
+      </c>
+      <c r="D40" s="13" t="inlineStr">
+        <is>
+          <t>39837694</t>
+        </is>
+      </c>
+      <c r="E40" s="13" t="inlineStr">
+        <is>
+          <t>10.1016/j.clbc.2024.12.015</t>
+        </is>
+      </c>
+      <c r="F40" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G40" s="15" t="inlineStr"/>
+      <c r="H40" s="15" t="inlineStr"/>
+      <c r="I40" s="16" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="13" t="inlineStr">
+        <is>
+          <t>474</t>
+        </is>
+      </c>
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C41" s="14" t="inlineStr">
+        <is>
+          <t>Persistent poverty and breast cancer incidence by tumor subtype: intersections of rural/urban residence and race within USA Surveillance Epidemiology and End Results Registries, 2017 to 2021 (2026)</t>
+        </is>
+      </c>
+      <c r="D41" s="13" t="inlineStr">
+        <is>
+          <t>41546752</t>
+        </is>
+      </c>
+      <c r="E41" s="13" t="inlineStr">
+        <is>
+          <t>10.1007/s10552-025-02114-z</t>
+        </is>
+      </c>
+      <c r="F41" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G41" s="15" t="inlineStr"/>
+      <c r="H41" s="15" t="inlineStr"/>
+      <c r="I41" s="16" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="13" t="inlineStr">
+        <is>
+          <t>477</t>
+        </is>
+      </c>
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C42" s="14" t="inlineStr">
+        <is>
+          <t>Spillover effects of public school integration in the southern United States: diverging trends in statewide annual breast cancer incidence, 2001–2019 (2026)</t>
+        </is>
+      </c>
+      <c r="D42" s="13" t="inlineStr">
+        <is>
+          <t>41649619</t>
+        </is>
+      </c>
+      <c r="E42" s="13" t="inlineStr">
+        <is>
+          <t>10.1007/s10552-025-02124-x</t>
+        </is>
+      </c>
+      <c r="F42" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G42" s="15" t="inlineStr"/>
+      <c r="H42" s="15" t="inlineStr"/>
+      <c r="I42" s="16" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="13" t="inlineStr">
+        <is>
+          <t>504</t>
+        </is>
+      </c>
+      <c r="B43" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C43" s="14" t="inlineStr">
+        <is>
+          <t>Cancer Incidence and Trends in Persistent Poverty Areas of California by Race/Ethnicity and Sex (2025)</t>
+        </is>
+      </c>
+      <c r="D43" s="13" t="inlineStr">
+        <is>
+          <t>40736150</t>
+        </is>
+      </c>
+      <c r="E43" s="13" t="inlineStr">
+        <is>
+          <t>10.1002/cam4.71088</t>
+        </is>
+      </c>
+      <c r="F43" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G43" s="15" t="inlineStr"/>
+      <c r="H43" s="15" t="inlineStr"/>
+      <c r="I43" s="16" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="13" t="inlineStr">
+        <is>
+          <t>510</t>
+        </is>
+      </c>
+      <c r="B44" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C44" s="14" t="inlineStr">
+        <is>
+          <t>Cancer statistics for Asian Americans, Native Hawaiians, and Pacific Islanders, 2016: Converging incidence in males and females (2016)</t>
+        </is>
+      </c>
+      <c r="D44" s="13" t="inlineStr">
+        <is>
+          <t>26766789</t>
+        </is>
+      </c>
+      <c r="E44" s="13" t="inlineStr">
+        <is>
+          <t>10.3322/caac.21335</t>
+        </is>
+      </c>
+      <c r="F44" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G44" s="15" t="inlineStr"/>
+      <c r="H44" s="15" t="inlineStr"/>
+      <c r="I44" s="16" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="13" t="inlineStr">
+        <is>
+          <t>516</t>
+        </is>
+      </c>
+      <c r="B45" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C45" s="14" t="inlineStr">
+        <is>
+          <t>The role of area-level socioeconomic disadvantage in racial disparities in cancer incidence in metropolitan Detroit (2023)</t>
+        </is>
+      </c>
+      <c r="D45" s="13" t="inlineStr">
+        <is>
+          <t>37184135</t>
+        </is>
+      </c>
+      <c r="E45" s="13" t="inlineStr">
+        <is>
+          <t>10.1002/cam4.6065</t>
+        </is>
+      </c>
+      <c r="F45" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G45" s="15" t="inlineStr"/>
+      <c r="H45" s="15" t="inlineStr"/>
+      <c r="I45" s="16" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="13" t="inlineStr">
+        <is>
+          <t>565</t>
+        </is>
+      </c>
+      <c r="B46" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C46" s="14" t="inlineStr">
+        <is>
+          <t>Cancer in Guam and Hawaii: A comparison of two U.S. Island populations (2017)</t>
+        </is>
+      </c>
+      <c r="D46" s="13" t="inlineStr">
+        <is>
+          <t>29120826</t>
+        </is>
+      </c>
+      <c r="E46" s="13" t="inlineStr">
+        <is>
+          <t>10.1016/j.canep.2017.08.005</t>
+        </is>
+      </c>
+      <c r="F46" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G46" s="15" t="inlineStr"/>
+      <c r="H46" s="15" t="inlineStr"/>
+      <c r="I46" s="16" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="13" t="inlineStr">
+        <is>
+          <t>751</t>
+        </is>
+      </c>
+      <c r="B47" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C47" s="14" t="inlineStr">
+        <is>
+          <t>Population-based statistics for women diagnosed with inflammatory breast cancer (United States) (2004)</t>
+        </is>
+      </c>
+      <c r="D47" s="13" t="inlineStr">
+        <is>
+          <t>15090727</t>
+        </is>
+      </c>
+      <c r="E47" s="13" t="inlineStr">
+        <is>
+          <t>10.1023/b:caco.0000024222.61114.18</t>
+        </is>
+      </c>
+      <c r="F47" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G47" s="15" t="inlineStr"/>
+      <c r="H47" s="15" t="inlineStr"/>
+      <c r="I47" s="16" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="13" t="inlineStr">
+        <is>
+          <t>754</t>
+        </is>
+      </c>
+      <c r="B48" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C48" s="14" t="inlineStr">
+        <is>
+          <t>Breast cancer incidence and stage at diagnosis in the six US-Affiliated Pacific  Islands (2024)</t>
+        </is>
+      </c>
+      <c r="D48" s="13" t="inlineStr">
+        <is>
+          <t>38996557</t>
+        </is>
+      </c>
+      <c r="E48" s="13" t="inlineStr">
+        <is>
+          <t>10.1016/j.canep.2024.102611</t>
+        </is>
+      </c>
+      <c r="F48" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G48" s="15" t="inlineStr"/>
+      <c r="H48" s="15" t="inlineStr"/>
+      <c r="I48" s="16" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="13" t="inlineStr">
+        <is>
+          <t>998</t>
+        </is>
+      </c>
+      <c r="B49" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C49" s="14" t="inlineStr">
+        <is>
+          <t>Cancer-related risk factors and incidence of major cancers by race, gender and region; analysis of the NIH-AARP diet and health study (2017)</t>
+        </is>
+      </c>
+      <c r="D49" s="13" t="inlineStr">
+        <is>
+          <t>28854891</t>
+        </is>
+      </c>
+      <c r="E49" s="13" t="inlineStr">
+        <is>
+          <t>10.1186/s12885-017-3557-1</t>
+        </is>
+      </c>
+      <c r="F49" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G49" s="15" t="inlineStr"/>
+      <c r="H49" s="15" t="inlineStr"/>
+      <c r="I49" s="16" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="13" t="inlineStr">
+        <is>
+          <t>1101</t>
+        </is>
+      </c>
+      <c r="B50" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C50" s="14" t="inlineStr">
+        <is>
+          <t>Cancer incidence in the Somali population of Olmsted County: A Rochester epidemiology project study (2023)</t>
+        </is>
+      </c>
+      <c r="D50" s="13" t="inlineStr">
+        <is>
+          <t>37740603</t>
+        </is>
+      </c>
+      <c r="E50" s="13" t="inlineStr">
+        <is>
+          <t>10.1002/cam4.6558</t>
+        </is>
+      </c>
+      <c r="F50" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G50" s="15" t="inlineStr"/>
+      <c r="H50" s="15" t="inlineStr"/>
+      <c r="I50" s="16" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="13" t="inlineStr">
+        <is>
+          <t>1398</t>
+        </is>
+      </c>
+      <c r="B51" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C51" s="14" t="inlineStr">
+        <is>
+          <t>Early-Onset Cancer Incidence Disparities Between Black and White Individuals in the US, 2003-2022 (2026)</t>
+        </is>
+      </c>
+      <c r="D51" s="13" t="inlineStr">
+        <is>
+          <t>41989785</t>
+        </is>
+      </c>
+      <c r="E51" s="13" t="inlineStr">
+        <is>
+          <t>10.1001/jamanetworkopen.2026.7529</t>
+        </is>
+      </c>
+      <c r="F51" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G51" s="15" t="inlineStr"/>
+      <c r="H51" s="15" t="inlineStr"/>
+      <c r="I51" s="16" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="13" t="inlineStr">
+        <is>
+          <t>1453</t>
+        </is>
+      </c>
+      <c r="B52" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C52" s="14" t="inlineStr">
+        <is>
+          <t>American Cancer Society’s Report on the Status of Cancer Disparities in the United States, 2025 (2026)</t>
+        </is>
+      </c>
+      <c r="D52" s="13" t="inlineStr">
+        <is>
+          <t>41400551</t>
+        </is>
+      </c>
+      <c r="E52" s="13" t="inlineStr">
+        <is>
+          <t>10.3322/caac.70045</t>
+        </is>
+      </c>
+      <c r="F52" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G52" s="15" t="inlineStr"/>
+      <c r="H52" s="15" t="inlineStr"/>
+      <c r="I52" s="16" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="13" t="inlineStr">
+        <is>
+          <t>1457</t>
+        </is>
+      </c>
+      <c r="B53" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C53" s="14" t="inlineStr">
+        <is>
+          <t>Cancer statistics, 2026 (2026)</t>
+        </is>
+      </c>
+      <c r="D53" s="13" t="inlineStr">
+        <is>
+          <t>41528114</t>
+        </is>
+      </c>
+      <c r="E53" s="13" t="inlineStr">
+        <is>
+          <t>10.3322/caac.70043</t>
+        </is>
+      </c>
+      <c r="F53" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G53" s="15" t="inlineStr"/>
+      <c r="H53" s="15" t="inlineStr"/>
+      <c r="I53" s="16" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="13" t="inlineStr">
+        <is>
+          <t>1569</t>
+        </is>
+      </c>
+      <c r="B54" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C54" s="14" t="inlineStr">
+        <is>
+          <t>Characterizing cancer patterns in Okinawan vs. mainland Japanese Americans: The Multiethnic Cohort Study (2025)</t>
+        </is>
+      </c>
+      <c r="D54" s="13" t="inlineStr"/>
+      <c r="E54" s="13" t="inlineStr">
+        <is>
+          <t>10.1101/2025.07.14.25331338</t>
+        </is>
+      </c>
+      <c r="F54" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G54" s="15" t="inlineStr"/>
+      <c r="H54" s="15" t="inlineStr"/>
+      <c r="I54" s="16" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="13" t="inlineStr">
+        <is>
+          <t>1629</t>
+        </is>
+      </c>
+      <c r="B55" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C55" s="14" t="inlineStr">
+        <is>
+          <t>Inequalities in Fertility-Impacting Cancer Incidence Among Young Populations in the United States (2025)</t>
+        </is>
+      </c>
+      <c r="D55" s="13" t="inlineStr">
+        <is>
+          <t>40189850</t>
+        </is>
+      </c>
+      <c r="E55" s="13" t="inlineStr">
+        <is>
+          <t>10.1002/cam4.70797</t>
+        </is>
+      </c>
+      <c r="F55" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G55" s="15" t="inlineStr"/>
+      <c r="H55" s="15" t="inlineStr"/>
+      <c r="I55" s="16" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="13" t="inlineStr">
+        <is>
+          <t>1637</t>
+        </is>
+      </c>
+      <c r="B56" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C56" s="14" t="inlineStr">
+        <is>
+          <t>Cancer Incidence in the Hispanic Community Health Study/Study of Latinos (HCHS/SOL)—The Onco-SOL Ancillary Study (2025)</t>
+        </is>
+      </c>
+      <c r="D56" s="13" t="inlineStr">
+        <is>
+          <t>39808161</t>
+        </is>
+      </c>
+      <c r="E56" s="13" t="inlineStr">
+        <is>
+          <t>10.1158/1055-9965.epi-24-1325</t>
+        </is>
+      </c>
+      <c r="F56" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G56" s="15" t="inlineStr"/>
+      <c r="H56" s="15" t="inlineStr"/>
+      <c r="I56" s="16" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="13" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="B57" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C57" s="14" t="inlineStr">
+        <is>
+          <t>Rural–Urban Cancer Incidence and Trends in the United States, 2000 to 2019 (2024)</t>
+        </is>
+      </c>
+      <c r="D57" s="13" t="inlineStr">
+        <is>
+          <t>38801414</t>
+        </is>
+      </c>
+      <c r="E57" s="13" t="inlineStr">
+        <is>
+          <t>10.1158/1055-9965.epi-24-0072</t>
+        </is>
+      </c>
+      <c r="F57" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G57" s="15" t="inlineStr"/>
+      <c r="H57" s="15" t="inlineStr"/>
+      <c r="I57" s="16" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="13" t="inlineStr">
+        <is>
+          <t>2440</t>
+        </is>
+      </c>
+      <c r="B58" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C58" s="14" t="inlineStr">
+        <is>
+          <t>Cancer incidence and associations with known risk and protective factors: the Alaska EARTH study (2019)</t>
+        </is>
+      </c>
+      <c r="D58" s="13" t="inlineStr">
+        <is>
+          <t>31428891</t>
+        </is>
+      </c>
+      <c r="E58" s="13" t="inlineStr">
+        <is>
+          <t>10.1007/s10552-019-01216-9</t>
+        </is>
+      </c>
+      <c r="F58" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G58" s="15" t="inlineStr"/>
+      <c r="H58" s="15" t="inlineStr"/>
+      <c r="I58" s="16" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="13" t="inlineStr">
+        <is>
+          <t>2453</t>
+        </is>
+      </c>
+      <c r="B59" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C59" s="14" t="inlineStr">
+        <is>
+          <t>Incidence and survival among young women with stage I-III breast cancer: Seer 2000-2015 (2019)</t>
+        </is>
+      </c>
+      <c r="D59" s="13" t="inlineStr">
+        <is>
+          <t>31392297</t>
+        </is>
+      </c>
+      <c r="E59" s="13" t="inlineStr">
+        <is>
+          <t>10.1093/jncics/pkz040</t>
+        </is>
+      </c>
+      <c r="F59" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G59" s="15" t="inlineStr"/>
+      <c r="H59" s="15" t="inlineStr"/>
+      <c r="I59" s="16" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="13" t="inlineStr">
+        <is>
+          <t>3845</t>
+        </is>
+      </c>
+      <c r="B60" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C60" s="14" t="inlineStr">
+        <is>
+          <t>Characterizing inflammatory breast cancer among Arab Americans in the California, Detroit and New Jersey Surveillance, Epidemiology and End Results (SEER) registries (1988-2008) (2013)</t>
+        </is>
+      </c>
+      <c r="D60" s="13" t="inlineStr"/>
+      <c r="E60" s="13" t="inlineStr">
+        <is>
+          <t>10.1186/2193-1801-2-3</t>
+        </is>
+      </c>
+      <c r="F60" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G60" s="15" t="inlineStr"/>
+      <c r="H60" s="15" t="inlineStr"/>
+      <c r="I60" s="16" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="13" t="inlineStr">
+        <is>
+          <t>4043</t>
+        </is>
+      </c>
+      <c r="B61" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C61" s="14" t="inlineStr">
+        <is>
+          <t>Trends in Breast Cancer Incidence and Mortality in the United States From 2004-2018: A Surveillance, Epidemiology, and End Results (SEER)-Based Study (2023)</t>
+        </is>
+      </c>
+      <c r="D61" s="13" t="inlineStr">
+        <is>
+          <t>37223193</t>
+        </is>
+      </c>
+      <c r="E61" s="13" t="inlineStr">
+        <is>
+          <t>10.7759/cureus.37982</t>
+        </is>
+      </c>
+      <c r="F61" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G61" s="15" t="inlineStr"/>
+      <c r="H61" s="15" t="inlineStr"/>
+      <c r="I61" s="16" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="13" t="inlineStr">
+        <is>
+          <t>4082</t>
+        </is>
+      </c>
+      <c r="B62" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C62" s="14" t="inlineStr">
+        <is>
+          <t>Annual Report to the Nation on the Status of Cancer, featuring state-level statistics after the onset of the COVID-19 pandemic (2025)</t>
+        </is>
+      </c>
+      <c r="D62" s="13" t="inlineStr">
+        <is>
+          <t>40257373</t>
+        </is>
+      </c>
+      <c r="E62" s="13" t="inlineStr">
+        <is>
+          <t>10.1002/cncr.35833</t>
+        </is>
+      </c>
+      <c r="F62" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G62" s="15" t="inlineStr"/>
+      <c r="H62" s="15" t="inlineStr"/>
+      <c r="I62" s="16" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="13" t="inlineStr">
+        <is>
+          <t>4294</t>
+        </is>
+      </c>
+      <c r="B63" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C63" s="14" t="inlineStr">
+        <is>
+          <t>Cancer statistics for African American and Black people, 2025 (2025)</t>
+        </is>
+      </c>
+      <c r="D63" s="13" t="inlineStr">
+        <is>
+          <t>39976243</t>
+        </is>
+      </c>
+      <c r="E63" s="13" t="inlineStr">
+        <is>
+          <t>10.3322/caac.21874</t>
+        </is>
+      </c>
+      <c r="F63" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G63" s="15" t="inlineStr"/>
+      <c r="H63" s="15" t="inlineStr"/>
+      <c r="I63" s="16" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="13" t="inlineStr">
+        <is>
+          <t>4389</t>
+        </is>
+      </c>
+      <c r="B64" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C64" s="14" t="inlineStr">
+        <is>
+          <t>Differences in the cancer burden among foreign-born and US-born Arab Americans living in metropolitan Detroit (2013)</t>
+        </is>
+      </c>
+      <c r="D64" s="13" t="inlineStr">
+        <is>
+          <t>24013772</t>
+        </is>
+      </c>
+      <c r="E64" s="13" t="inlineStr">
+        <is>
+          <t>10.1007/s10552-013-0271-4</t>
+        </is>
+      </c>
+      <c r="F64" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G64" s="15" t="inlineStr"/>
+      <c r="H64" s="15" t="inlineStr"/>
+      <c r="I64" s="16" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="13" t="inlineStr">
+        <is>
+          <t>4429</t>
+        </is>
+      </c>
+      <c r="B65" s="13" t="inlineStr">
+        <is>
+          <t>INCLUDED (narrative)</t>
+        </is>
+      </c>
+      <c r="C65" s="14" t="inlineStr">
+        <is>
+          <t>Cancer risk in different generations of Middle Eastern immigrants to California, 1988-2013 (2017)</t>
+        </is>
+      </c>
+      <c r="D65" s="13" t="inlineStr">
+        <is>
+          <t>28801942</t>
+        </is>
+      </c>
+      <c r="E65" s="13" t="inlineStr">
+        <is>
+          <t>10.1002/ijc.30928</t>
+        </is>
+      </c>
+      <c r="F65" s="14" t="inlineStr">
+        <is>
+          <t>LOW — narrative only</t>
+        </is>
+      </c>
+      <c r="G65" s="15" t="inlineStr"/>
+      <c r="H65" s="15" t="inlineStr"/>
+      <c r="I65" s="16" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="13" t="inlineStr">
+        <is>
+          <t>1462</t>
+        </is>
+      </c>
+      <c r="B66" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Ineligible population)</t>
+        </is>
+      </c>
+      <c r="C66" s="14" t="inlineStr">
+        <is>
+          <t>Rising Breast Cancer Incidence and Poor Outcomes in Young Women: A Retrospective Study (2026)</t>
+        </is>
+      </c>
+      <c r="D66" s="13" t="inlineStr">
+        <is>
+          <t>41742962</t>
+        </is>
+      </c>
+      <c r="E66" s="13" t="inlineStr">
+        <is>
+          <t>10.1155/tbj/5584726</t>
+        </is>
+      </c>
+      <c r="F66" s="14" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="G66" s="15" t="inlineStr"/>
+      <c r="H66" s="15" t="inlineStr"/>
+      <c r="I66" s="16" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B67" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
+        </is>
+      </c>
+      <c r="C67" s="14" t="inlineStr">
+        <is>
+          <t>Lobular breast cancer statistics, 2025 (2025)</t>
+        </is>
+      </c>
+      <c r="D67" s="13" t="inlineStr">
+        <is>
+          <t>41055508</t>
+        </is>
+      </c>
+      <c r="E67" s="13" t="inlineStr">
+        <is>
+          <t>10.1002/cncr.70061</t>
+        </is>
+      </c>
+      <c r="F67" s="14" t="inlineStr">
+        <is>
+          <t>LOW — metadata-defensible</t>
+        </is>
+      </c>
+      <c r="G67" s="15" t="inlineStr"/>
+      <c r="H67" s="15" t="inlineStr"/>
+      <c r="I67" s="16" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="13" t="inlineStr">
+        <is>
+          <t>156</t>
+        </is>
+      </c>
+      <c r="B68" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
+        </is>
+      </c>
+      <c r="C68" s="14" t="inlineStr">
+        <is>
+          <t>Annual report to the nation on the status of cancer, part 1: National cancer statistics (2022)</t>
+        </is>
+      </c>
+      <c r="D68" s="13" t="inlineStr">
+        <is>
+          <t>36301149</t>
+        </is>
+      </c>
+      <c r="E68" s="13" t="inlineStr">
+        <is>
+          <t>10.1002/cncr.34479</t>
+        </is>
+      </c>
+      <c r="F68" s="14" t="inlineStr">
+        <is>
+          <t>LOW — metadata-defensible</t>
+        </is>
+      </c>
+      <c r="G68" s="15" t="inlineStr"/>
+      <c r="H68" s="15" t="inlineStr"/>
+      <c r="I68" s="16" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="13" t="inlineStr">
+        <is>
+          <t>235</t>
+        </is>
+      </c>
+      <c r="B69" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
+        </is>
+      </c>
+      <c r="C69" s="14" t="inlineStr">
+        <is>
+          <t>Annual report to the nation on the status of cancer, part I: National cancer statistics (2020)</t>
+        </is>
+      </c>
+      <c r="D69" s="13" t="inlineStr">
+        <is>
+          <t>32162336</t>
+        </is>
+      </c>
+      <c r="E69" s="13" t="inlineStr">
+        <is>
+          <t>10.1002/cncr.32802</t>
+        </is>
+      </c>
+      <c r="F69" s="14" t="inlineStr">
+        <is>
+          <t>LOW — metadata-defensible</t>
+        </is>
+      </c>
+      <c r="G69" s="15" t="inlineStr"/>
+      <c r="H69" s="15" t="inlineStr"/>
+      <c r="I69" s="16" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="13" t="inlineStr">
+        <is>
+          <t>358</t>
+        </is>
+      </c>
+      <c r="B70" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
+        </is>
+      </c>
+      <c r="C70" s="14" t="inlineStr">
+        <is>
+          <t>Annual Report to the Nation on the status of cancer, 1975-2010, featuring  prevalence of comorbidity and impact on survival among persons with lung, colorectal, breast, or prostate cancer (2014)</t>
+        </is>
+      </c>
+      <c r="D70" s="13" t="inlineStr">
+        <is>
+          <t>24343171</t>
+        </is>
+      </c>
+      <c r="E70" s="13" t="inlineStr">
+        <is>
+          <t>10.1002/cncr.28509</t>
+        </is>
+      </c>
+      <c r="F70" s="14" t="inlineStr">
+        <is>
+          <t>LOW — metadata-defensible</t>
+        </is>
+      </c>
+      <c r="G70" s="15" t="inlineStr"/>
+      <c r="H70" s="15" t="inlineStr"/>
+      <c r="I70" s="16" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="13" t="inlineStr">
+        <is>
+          <t>362</t>
+        </is>
+      </c>
+      <c r="B71" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
+        </is>
+      </c>
+      <c r="C71" s="14" t="inlineStr">
+        <is>
+          <t>Annual Report to the Nation on the Status of Cancer, 1975-2014, Featuring  Survival (2017)</t>
+        </is>
+      </c>
+      <c r="D71" s="13" t="inlineStr">
+        <is>
+          <t>28376154</t>
+        </is>
+      </c>
+      <c r="E71" s="13" t="inlineStr">
+        <is>
+          <t>10.1093/jnci/djx030</t>
+        </is>
+      </c>
+      <c r="F71" s="14" t="inlineStr">
+        <is>
+          <t>LOW — metadata-defensible</t>
+        </is>
+      </c>
+      <c r="G71" s="15" t="inlineStr"/>
+      <c r="H71" s="15" t="inlineStr"/>
+      <c r="I71" s="16" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="13" t="inlineStr">
+        <is>
+          <t>384</t>
+        </is>
+      </c>
+      <c r="B72" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
+        </is>
+      </c>
+      <c r="C72" s="14" t="inlineStr">
+        <is>
+          <t>Annual report to the nation on the status of cancer, 1975-2003, featuring cancer  among U.S. Hispanic/Latino populations (2006)</t>
+        </is>
+      </c>
+      <c r="D72" s="13" t="inlineStr">
+        <is>
+          <t>16958083</t>
+        </is>
+      </c>
+      <c r="E72" s="13" t="inlineStr">
+        <is>
+          <t>10.1002/cncr.22193</t>
+        </is>
+      </c>
+      <c r="F72" s="14" t="inlineStr">
+        <is>
+          <t>LOW — metadata-defensible</t>
+        </is>
+      </c>
+      <c r="G72" s="15" t="inlineStr"/>
+      <c r="H72" s="15" t="inlineStr"/>
+      <c r="I72" s="16" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="13" t="inlineStr">
+        <is>
+          <t>411</t>
+        </is>
+      </c>
+      <c r="B73" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
+        </is>
+      </c>
+      <c r="C73" s="14" t="inlineStr">
+        <is>
+          <t>Annual report to the nation on the status of cancer, 1975-2011, featuring incidence of breast cancer subtypes by race/ethnicity, poverty, and state (2015)</t>
+        </is>
+      </c>
+      <c r="D73" s="13" t="inlineStr">
+        <is>
+          <t>25825511</t>
+        </is>
+      </c>
+      <c r="E73" s="13" t="inlineStr">
+        <is>
+          <t>10.1093/jnci/djv048</t>
+        </is>
+      </c>
+      <c r="F73" s="14" t="inlineStr">
+        <is>
+          <t>LOW — metadata-defensible</t>
+        </is>
+      </c>
+      <c r="G73" s="15" t="inlineStr"/>
+      <c r="H73" s="15" t="inlineStr"/>
+      <c r="I73" s="16" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="13" t="inlineStr">
+        <is>
+          <t>788</t>
+        </is>
+      </c>
+      <c r="B74" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
+        </is>
+      </c>
+      <c r="C74" s="14" t="inlineStr">
+        <is>
+          <t>Annual Report to the Nation on the Status of Cancer, Featuring Cancer in Men and Women Age 20–49 Years (2019)</t>
+        </is>
+      </c>
+      <c r="D74" s="13" t="inlineStr">
+        <is>
+          <t>31145458</t>
+        </is>
+      </c>
+      <c r="E74" s="13" t="inlineStr">
+        <is>
+          <t>10.1093/jnci/djz106</t>
+        </is>
+      </c>
+      <c r="F74" s="14" t="inlineStr">
+        <is>
+          <t>LOW — metadata-defensible</t>
+        </is>
+      </c>
+      <c r="G74" s="15" t="inlineStr"/>
+      <c r="H74" s="15" t="inlineStr"/>
+      <c r="I74" s="16" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="13" t="inlineStr">
+        <is>
+          <t>968</t>
+        </is>
+      </c>
+      <c r="B75" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
+        </is>
+      </c>
+      <c r="C75" s="14" t="inlineStr">
+        <is>
+          <t>Annual report to the nation on the status of cancer, 1975-2006, featuring  colorectal cancer trends and impact of interventions (risk factors, screening, and treatment) to reduce future rates (2010)</t>
+        </is>
+      </c>
+      <c r="D75" s="13" t="inlineStr">
+        <is>
+          <t>19998273</t>
+        </is>
+      </c>
+      <c r="E75" s="13" t="inlineStr">
+        <is>
+          <t>10.1002/cncr.24760</t>
+        </is>
+      </c>
+      <c r="F75" s="14" t="inlineStr">
+        <is>
+          <t>LOW — metadata-defensible</t>
+        </is>
+      </c>
+      <c r="G75" s="15" t="inlineStr"/>
+      <c r="H75" s="15" t="inlineStr"/>
+      <c r="I75" s="16" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="13" t="inlineStr">
+        <is>
+          <t>2151</t>
+        </is>
+      </c>
+      <c r="B76" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
+        </is>
+      </c>
+      <c r="C76" s="14" t="inlineStr">
+        <is>
+          <t>American Cancer Society's report on the status of cancer disparities in the United States, 2021 (2022)</t>
+        </is>
+      </c>
+      <c r="D76" s="13" t="inlineStr">
+        <is>
+          <t>34878180</t>
+        </is>
+      </c>
+      <c r="E76" s="13" t="inlineStr">
+        <is>
+          <t>10.3322/caac.21703</t>
+        </is>
+      </c>
+      <c r="F76" s="14" t="inlineStr">
+        <is>
+          <t>LOW — metadata-defensible</t>
+        </is>
+      </c>
+      <c r="G76" s="15" t="inlineStr"/>
+      <c r="H76" s="15" t="inlineStr"/>
+      <c r="I76" s="16" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="13" t="inlineStr">
+        <is>
+          <t>2163</t>
+        </is>
+      </c>
+      <c r="B77" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
+        </is>
+      </c>
+      <c r="C77" s="14" t="inlineStr">
+        <is>
+          <t>Estrogen receptor negative breast cancer incidence rates are similar in Ghanaian and Non-Hispanic Black women in the USA (2022)</t>
+        </is>
+      </c>
+      <c r="D77" s="13" t="inlineStr"/>
+      <c r="E77" s="13" t="inlineStr">
+        <is>
+          <t>10.1101/2022.02.21.22271266</t>
+        </is>
+      </c>
+      <c r="F77" s="14" t="inlineStr">
+        <is>
+          <t>LOW — metadata-defensible</t>
+        </is>
+      </c>
+      <c r="G77" s="15" t="inlineStr"/>
+      <c r="H77" s="15" t="inlineStr"/>
+      <c r="I77" s="16" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="13" t="inlineStr">
+        <is>
+          <t>3373</t>
+        </is>
+      </c>
+      <c r="B78" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
+        </is>
+      </c>
+      <c r="C78" s="14" t="inlineStr">
+        <is>
+          <t>Cancer Statistics, 2004 (2004)</t>
+        </is>
+      </c>
+      <c r="D78" s="13" t="inlineStr">
+        <is>
+          <t>14974761</t>
+        </is>
+      </c>
+      <c r="E78" s="13" t="inlineStr">
+        <is>
+          <t>10.3322/canjclin.54.1.8</t>
+        </is>
+      </c>
+      <c r="F78" s="14" t="inlineStr">
+        <is>
+          <t>LOW — metadata-defensible</t>
+        </is>
+      </c>
+      <c r="G78" s="15" t="inlineStr"/>
+      <c r="H78" s="15" t="inlineStr"/>
+      <c r="I78" s="16" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="13" t="inlineStr">
+        <is>
+          <t>3429</t>
+        </is>
+      </c>
+      <c r="B79" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
+        </is>
+      </c>
+      <c r="C79" s="14" t="inlineStr">
+        <is>
+          <t>Cancer statistics, 2002 (2002)</t>
+        </is>
+      </c>
+      <c r="D79" s="13" t="inlineStr">
+        <is>
+          <t>11814064</t>
+        </is>
+      </c>
+      <c r="E79" s="13" t="inlineStr">
+        <is>
+          <t>10.3322/canjclin.52.1.23</t>
+        </is>
+      </c>
+      <c r="F79" s="14" t="inlineStr">
+        <is>
+          <t>LOW — metadata-defensible</t>
+        </is>
+      </c>
+      <c r="G79" s="15" t="inlineStr"/>
+      <c r="H79" s="15" t="inlineStr"/>
+      <c r="I79" s="16" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="13" t="inlineStr">
+        <is>
+          <t>3522</t>
+        </is>
+      </c>
+      <c r="B80" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
+        </is>
+      </c>
+      <c r="C80" s="14" t="inlineStr">
+        <is>
+          <t>Annual Report to the Nation on the Status of Cancer, part 2: Early assessment of the COVID-19 pandemic’s impact on cancer diagnosis (2024)</t>
+        </is>
+      </c>
+      <c r="D80" s="13" t="inlineStr"/>
+      <c r="E80" s="13" t="inlineStr">
+        <is>
+          <t>10.1002/cncr.35026</t>
+        </is>
+      </c>
+      <c r="F80" s="14" t="inlineStr">
+        <is>
+          <t>LOW — metadata-defensible</t>
+        </is>
+      </c>
+      <c r="G80" s="15" t="inlineStr"/>
+      <c r="H80" s="15" t="inlineStr"/>
+      <c r="I80" s="16" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="13" t="inlineStr">
+        <is>
+          <t>3713</t>
+        </is>
+      </c>
+      <c r="B81" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
+        </is>
+      </c>
+      <c r="C81" s="14" t="inlineStr">
+        <is>
+          <t>Cancer incidence and mortality among Filipinos in the USA and the Philippines: Patterns and trends (2016)</t>
+        </is>
+      </c>
+      <c r="D81" s="13" t="inlineStr"/>
+      <c r="E81" s="13" t="inlineStr">
+        <is>
+          <t>10.1007/978-3-319-41118-7_3</t>
+        </is>
+      </c>
+      <c r="F81" s="14" t="inlineStr">
+        <is>
+          <t>LOW — metadata-defensible</t>
+        </is>
+      </c>
+      <c r="G81" s="15" t="inlineStr"/>
+      <c r="H81" s="15" t="inlineStr"/>
+      <c r="I81" s="16" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="13" t="inlineStr">
+        <is>
+          <t>4035</t>
+        </is>
+      </c>
+      <c r="B82" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
+        </is>
+      </c>
+      <c r="C82" s="14" t="inlineStr">
+        <is>
+          <t>Annual report to the nation on the status of cancer, 1975-2001, with a special feature regarding survival (2004)</t>
+        </is>
+      </c>
+      <c r="D82" s="13" t="inlineStr">
+        <is>
+          <t>15221985</t>
+        </is>
+      </c>
+      <c r="E82" s="13" t="inlineStr">
+        <is>
+          <t>10.1002/cncr.20288</t>
+        </is>
+      </c>
+      <c r="F82" s="14" t="inlineStr">
+        <is>
+          <t>LOW — metadata-defensible</t>
+        </is>
+      </c>
+      <c r="G82" s="15" t="inlineStr"/>
+      <c r="H82" s="15" t="inlineStr"/>
+      <c r="I82" s="16" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="13" t="inlineStr">
+        <is>
+          <t>4050</t>
+        </is>
+      </c>
+      <c r="B83" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
+        </is>
+      </c>
+      <c r="C83" s="14" t="inlineStr">
+        <is>
+          <t>Annual Report to the Nation on the Status of Cancer, 19752009, Featuring the Burden and Trends in Human Papillomavirus (HPV)Associated Cancers and HPV Vaccination Coverage Levels (2013)</t>
+        </is>
+      </c>
+      <c r="D83" s="13" t="inlineStr">
+        <is>
+          <t>23297039</t>
+        </is>
+      </c>
+      <c r="E83" s="13" t="inlineStr">
+        <is>
+          <t>10.1093/jnci/djs491</t>
+        </is>
+      </c>
+      <c r="F83" s="14" t="inlineStr">
+        <is>
+          <t>LOW — metadata-defensible</t>
+        </is>
+      </c>
+      <c r="G83" s="15" t="inlineStr"/>
+      <c r="H83" s="15" t="inlineStr"/>
+      <c r="I83" s="16" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="13" t="inlineStr">
+        <is>
+          <t>4057</t>
+        </is>
+      </c>
+      <c r="B84" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
+        </is>
+      </c>
+      <c r="C84" s="14" t="inlineStr">
+        <is>
+          <t>Breast cancer statistics, 2011 (2011)</t>
+        </is>
+      </c>
+      <c r="D84" s="13" t="inlineStr">
+        <is>
+          <t>21969133</t>
+        </is>
+      </c>
+      <c r="E84" s="13" t="inlineStr">
+        <is>
+          <t>10.3322/caac.20134</t>
+        </is>
+      </c>
+      <c r="F84" s="14" t="inlineStr">
+        <is>
+          <t>LOW — metadata-defensible</t>
+        </is>
+      </c>
+      <c r="G84" s="15" t="inlineStr"/>
+      <c r="H84" s="15" t="inlineStr"/>
+      <c r="I84" s="16" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="13" t="inlineStr">
+        <is>
+          <t>4065</t>
+        </is>
+      </c>
+      <c r="B85" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
+        </is>
+      </c>
+      <c r="C85" s="14" t="inlineStr">
+        <is>
+          <t>Cancer Statistics, 2014 (2014)</t>
+        </is>
+      </c>
+      <c r="D85" s="13" t="inlineStr">
+        <is>
+          <t>24399786</t>
+        </is>
+      </c>
+      <c r="E85" s="13" t="inlineStr">
+        <is>
+          <t>10.3322/caac.21208</t>
+        </is>
+      </c>
+      <c r="F85" s="14" t="inlineStr">
+        <is>
+          <t>LOW — metadata-defensible</t>
+        </is>
+      </c>
+      <c r="G85" s="15" t="inlineStr"/>
+      <c r="H85" s="15" t="inlineStr"/>
+      <c r="I85" s="16" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="13" t="inlineStr">
+        <is>
+          <t>4066</t>
+        </is>
+      </c>
+      <c r="B86" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
+        </is>
+      </c>
+      <c r="C86" s="14" t="inlineStr">
+        <is>
+          <t>Annual Report to the Nation on the Status of Cancer, 1975-2007, Featuring Tumors of the Brain and Other Nervous System (2011)</t>
+        </is>
+      </c>
+      <c r="D86" s="13" t="inlineStr">
+        <is>
+          <t>21454908</t>
+        </is>
+      </c>
+      <c r="E86" s="13" t="inlineStr">
+        <is>
+          <t>10.1093/jnci/djr077</t>
+        </is>
+      </c>
+      <c r="F86" s="14" t="inlineStr">
+        <is>
+          <t>LOW — metadata-defensible</t>
+        </is>
+      </c>
+      <c r="G86" s="15" t="inlineStr"/>
+      <c r="H86" s="15" t="inlineStr"/>
+      <c r="I86" s="16" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="13" t="inlineStr">
+        <is>
+          <t>4071</t>
+        </is>
+      </c>
+      <c r="B87" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
+        </is>
+      </c>
+      <c r="C87" s="14" t="inlineStr">
+        <is>
+          <t>Annual report to the nation on the status of cancer, 1975-2000, featuring the uses of surveillance data for cancer prevention and control (2003)</t>
+        </is>
+      </c>
+      <c r="D87" s="13" t="inlineStr">
+        <is>
+          <t>12953083</t>
+        </is>
+      </c>
+      <c r="E87" s="13" t="inlineStr">
+        <is>
+          <t>10.1093/jnci/djg040</t>
+        </is>
+      </c>
+      <c r="F87" s="14" t="inlineStr">
+        <is>
+          <t>LOW — metadata-defensible</t>
+        </is>
+      </c>
+      <c r="G87" s="15" t="inlineStr"/>
+      <c r="H87" s="15" t="inlineStr"/>
+      <c r="I87" s="16" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="13" t="inlineStr">
+        <is>
+          <t>4164</t>
+        </is>
+      </c>
+      <c r="B88" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
+        </is>
+      </c>
+      <c r="C88" s="14" t="inlineStr">
+        <is>
+          <t>Annual Report to the Nation on the Status of Cancer, 1975-2005, Featuring Trends in Lung Cancer, Tobacco Use, and Tobacco Control (2008)</t>
+        </is>
+      </c>
+      <c r="D88" s="13" t="inlineStr">
+        <is>
+          <t>19033571</t>
+        </is>
+      </c>
+      <c r="E88" s="13" t="inlineStr">
+        <is>
+          <t>10.1093/jnci/djn389</t>
+        </is>
+      </c>
+      <c r="F88" s="14" t="inlineStr">
+        <is>
+          <t>LOW — metadata-defensible</t>
+        </is>
+      </c>
+      <c r="G88" s="15" t="inlineStr"/>
+      <c r="H88" s="15" t="inlineStr"/>
+      <c r="I88" s="16" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="13" t="inlineStr">
+        <is>
+          <t>4172</t>
+        </is>
+      </c>
+      <c r="B89" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
+        </is>
+      </c>
+      <c r="C89" s="14" t="inlineStr">
+        <is>
+          <t>Cancer statistics, 2013 (2013)</t>
+        </is>
+      </c>
+      <c r="D89" s="13" t="inlineStr">
+        <is>
+          <t>23335087</t>
+        </is>
+      </c>
+      <c r="E89" s="13" t="inlineStr">
+        <is>
+          <t>10.3322/caac.21166</t>
+        </is>
+      </c>
+      <c r="F89" s="14" t="inlineStr">
+        <is>
+          <t>LOW — metadata-defensible</t>
+        </is>
+      </c>
+      <c r="G89" s="15" t="inlineStr"/>
+      <c r="H89" s="15" t="inlineStr"/>
+      <c r="I89" s="16" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="13" t="inlineStr">
+        <is>
+          <t>4213</t>
+        </is>
+      </c>
+      <c r="B90" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
+        </is>
+      </c>
+      <c r="C90" s="14" t="inlineStr">
+        <is>
+          <t>Cancer statistics for Hispanics/Latinos, 2012 (2012)</t>
+        </is>
+      </c>
+      <c r="D90" s="13" t="inlineStr">
+        <is>
+          <t>22987332</t>
+        </is>
+      </c>
+      <c r="E90" s="13" t="inlineStr">
+        <is>
+          <t>10.3322/caac.21153</t>
+        </is>
+      </c>
+      <c r="F90" s="14" t="inlineStr">
+        <is>
+          <t>LOW — metadata-defensible</t>
+        </is>
+      </c>
+      <c r="G90" s="15" t="inlineStr"/>
+      <c r="H90" s="15" t="inlineStr"/>
+      <c r="I90" s="16" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="13" t="inlineStr">
+        <is>
+          <t>4216</t>
+        </is>
+      </c>
+      <c r="B91" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
+        </is>
+      </c>
+      <c r="C91" s="14" t="inlineStr">
+        <is>
+          <t>Annual Report to the Nation on the status of cancer, 1975-2008, featuring cancers associated with excess weight and lack of sufficient physical activity (2012)</t>
+        </is>
+      </c>
+      <c r="D91" s="13" t="inlineStr">
+        <is>
+          <t>22460733</t>
+        </is>
+      </c>
+      <c r="E91" s="13" t="inlineStr">
+        <is>
+          <t>10.1002/cncr.27514</t>
+        </is>
+      </c>
+      <c r="F91" s="14" t="inlineStr">
+        <is>
+          <t>LOW — metadata-defensible</t>
+        </is>
+      </c>
+      <c r="G91" s="15" t="inlineStr"/>
+      <c r="H91" s="15" t="inlineStr"/>
+      <c r="I91" s="16" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="13" t="inlineStr">
+        <is>
+          <t>4357</t>
+        </is>
+      </c>
+      <c r="B92" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
+        </is>
+      </c>
+      <c r="C92" s="14" t="inlineStr">
+        <is>
+          <t>Cancer statistics for Hispanics, 2003 (2003)</t>
+        </is>
+      </c>
+      <c r="D92" s="13" t="inlineStr">
+        <is>
+          <t>12924775</t>
+        </is>
+      </c>
+      <c r="E92" s="13" t="inlineStr">
+        <is>
+          <t>10.3322/canjclin.53.4.208</t>
+        </is>
+      </c>
+      <c r="F92" s="14" t="inlineStr">
+        <is>
+          <t>LOW — metadata-defensible</t>
+        </is>
+      </c>
+      <c r="G92" s="15" t="inlineStr"/>
+      <c r="H92" s="15" t="inlineStr"/>
+      <c r="I92" s="16" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I92"/>
+  <dataValidations count="2">
+    <dataValidation sqref="G3:G92" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H3:H92" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Include,Exclude"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Classify 3 author-supplied PDFs (474/477/504) — all narrative, no upgrade
474 Sherr 2026 (SEER subtype, persistent-poverty rate differences; race = county
racial composition, ecological — no race-vs-NHW subtype IRR).
477 Chanpura 2026 (school-integration natural experiment; segmented-regression
trend among NHB/NHW birth cohorts, not an all-age race-vs-NHW IRR).
504 Movsisyan Vernon 2025 (California PPA-vs-nonPPA IRRs within race strata across
16 cancers; breast IRR is poverty-area contrast, not minority-vs-NHW; CCR overlap).

Reasons in outputs/Reclassification_log.md; workbook Sheet 6 (to-obtain) now 26.
78 cells, headline results, and crosschecks A-F unchanged.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CuLT4FKRBtsU22Vwfjj2qn
</commit_message>
<xml_diff>
--- a/meta_agents/search_v2/outputs/Author_Validation_Workbook.xlsx
+++ b/meta_agents/search_v2/outputs/Author_Validation_Workbook.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'2_TA_Excluded_Sample'!$A$1:$E$152</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'3_Extraction_Verification'!$A$1:$M$147</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'4_RoB_Review'!$A$1:$Q$45</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'6_FullText_ToObtain'!$A$1:$I$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'6_FullText_ToObtain'!$A$1:$I$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -23574,7 +23574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -24135,7 +24135,7 @@
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>474</t>
+          <t>510</t>
         </is>
       </c>
       <c r="B17" s="13" t="inlineStr">
@@ -24145,17 +24145,17 @@
       </c>
       <c r="C17" s="14" t="inlineStr">
         <is>
-          <t>Persistent poverty and breast cancer incidence by tumor subtype: intersections of rural/urban residence and race within USA Surveillance Epidemiology and End Results Registries, 2017 to 2021 (2026)</t>
+          <t>Cancer statistics for Asian Americans, Native Hawaiians, and Pacific Islanders, 2016: Converging incidence in males and females (2016)</t>
         </is>
       </c>
       <c r="D17" s="13" t="inlineStr">
         <is>
-          <t>41546752</t>
+          <t>26766789</t>
         </is>
       </c>
       <c r="E17" s="13" t="inlineStr">
         <is>
-          <t>10.1007/s10552-025-02114-z</t>
+          <t>10.3322/caac.21335</t>
         </is>
       </c>
       <c r="F17" s="14" t="inlineStr">
@@ -24170,7 +24170,7 @@
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
         <is>
-          <t>477</t>
+          <t>516</t>
         </is>
       </c>
       <c r="B18" s="13" t="inlineStr">
@@ -24180,17 +24180,17 @@
       </c>
       <c r="C18" s="14" t="inlineStr">
         <is>
-          <t>Spillover effects of public school integration in the southern United States: diverging trends in statewide annual breast cancer incidence, 2001–2019 (2026)</t>
+          <t>The role of area-level socioeconomic disadvantage in racial disparities in cancer incidence in metropolitan Detroit (2023)</t>
         </is>
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>41649619</t>
+          <t>37184135</t>
         </is>
       </c>
       <c r="E18" s="13" t="inlineStr">
         <is>
-          <t>10.1007/s10552-025-02124-x</t>
+          <t>10.1002/cam4.6065</t>
         </is>
       </c>
       <c r="F18" s="14" t="inlineStr">
@@ -24205,7 +24205,7 @@
     <row r="19">
       <c r="A19" s="13" t="inlineStr">
         <is>
-          <t>504</t>
+          <t>565</t>
         </is>
       </c>
       <c r="B19" s="13" t="inlineStr">
@@ -24215,17 +24215,17 @@
       </c>
       <c r="C19" s="14" t="inlineStr">
         <is>
-          <t>Cancer Incidence and Trends in Persistent Poverty Areas of California by Race/Ethnicity and Sex (2025)</t>
+          <t>Cancer in Guam and Hawaii: A comparison of two U.S. Island populations (2017)</t>
         </is>
       </c>
       <c r="D19" s="13" t="inlineStr">
         <is>
-          <t>40736150</t>
+          <t>29120826</t>
         </is>
       </c>
       <c r="E19" s="13" t="inlineStr">
         <is>
-          <t>10.1002/cam4.71088</t>
+          <t>10.1016/j.canep.2017.08.005</t>
         </is>
       </c>
       <c r="F19" s="14" t="inlineStr">
@@ -24240,7 +24240,7 @@
     <row r="20">
       <c r="A20" s="13" t="inlineStr">
         <is>
-          <t>510</t>
+          <t>751</t>
         </is>
       </c>
       <c r="B20" s="13" t="inlineStr">
@@ -24250,17 +24250,17 @@
       </c>
       <c r="C20" s="14" t="inlineStr">
         <is>
-          <t>Cancer statistics for Asian Americans, Native Hawaiians, and Pacific Islanders, 2016: Converging incidence in males and females (2016)</t>
+          <t>Population-based statistics for women diagnosed with inflammatory breast cancer (United States) (2004)</t>
         </is>
       </c>
       <c r="D20" s="13" t="inlineStr">
         <is>
-          <t>26766789</t>
+          <t>15090727</t>
         </is>
       </c>
       <c r="E20" s="13" t="inlineStr">
         <is>
-          <t>10.3322/caac.21335</t>
+          <t>10.1023/b:caco.0000024222.61114.18</t>
         </is>
       </c>
       <c r="F20" s="14" t="inlineStr">
@@ -24275,7 +24275,7 @@
     <row r="21">
       <c r="A21" s="13" t="inlineStr">
         <is>
-          <t>516</t>
+          <t>754</t>
         </is>
       </c>
       <c r="B21" s="13" t="inlineStr">
@@ -24285,17 +24285,17 @@
       </c>
       <c r="C21" s="14" t="inlineStr">
         <is>
-          <t>The role of area-level socioeconomic disadvantage in racial disparities in cancer incidence in metropolitan Detroit (2023)</t>
+          <t>Breast cancer incidence and stage at diagnosis in the six US-Affiliated Pacific  Islands (2024)</t>
         </is>
       </c>
       <c r="D21" s="13" t="inlineStr">
         <is>
-          <t>37184135</t>
+          <t>38996557</t>
         </is>
       </c>
       <c r="E21" s="13" t="inlineStr">
         <is>
-          <t>10.1002/cam4.6065</t>
+          <t>10.1016/j.canep.2024.102611</t>
         </is>
       </c>
       <c r="F21" s="14" t="inlineStr">
@@ -24310,7 +24310,7 @@
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
         <is>
-          <t>565</t>
+          <t>998</t>
         </is>
       </c>
       <c r="B22" s="13" t="inlineStr">
@@ -24320,17 +24320,17 @@
       </c>
       <c r="C22" s="14" t="inlineStr">
         <is>
-          <t>Cancer in Guam and Hawaii: A comparison of two U.S. Island populations (2017)</t>
+          <t>Cancer-related risk factors and incidence of major cancers by race, gender and region; analysis of the NIH-AARP diet and health study (2017)</t>
         </is>
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
-          <t>29120826</t>
+          <t>28854891</t>
         </is>
       </c>
       <c r="E22" s="13" t="inlineStr">
         <is>
-          <t>10.1016/j.canep.2017.08.005</t>
+          <t>10.1186/s12885-017-3557-1</t>
         </is>
       </c>
       <c r="F22" s="14" t="inlineStr">
@@ -24345,7 +24345,7 @@
     <row r="23">
       <c r="A23" s="13" t="inlineStr">
         <is>
-          <t>751</t>
+          <t>1101</t>
         </is>
       </c>
       <c r="B23" s="13" t="inlineStr">
@@ -24355,17 +24355,17 @@
       </c>
       <c r="C23" s="14" t="inlineStr">
         <is>
-          <t>Population-based statistics for women diagnosed with inflammatory breast cancer (United States) (2004)</t>
+          <t>Cancer incidence in the Somali population of Olmsted County: A Rochester epidemiology project study (2023)</t>
         </is>
       </c>
       <c r="D23" s="13" t="inlineStr">
         <is>
-          <t>15090727</t>
+          <t>37740603</t>
         </is>
       </c>
       <c r="E23" s="13" t="inlineStr">
         <is>
-          <t>10.1023/b:caco.0000024222.61114.18</t>
+          <t>10.1002/cam4.6558</t>
         </is>
       </c>
       <c r="F23" s="14" t="inlineStr">
@@ -24380,7 +24380,7 @@
     <row r="24">
       <c r="A24" s="13" t="inlineStr">
         <is>
-          <t>754</t>
+          <t>1398</t>
         </is>
       </c>
       <c r="B24" s="13" t="inlineStr">
@@ -24390,17 +24390,17 @@
       </c>
       <c r="C24" s="14" t="inlineStr">
         <is>
-          <t>Breast cancer incidence and stage at diagnosis in the six US-Affiliated Pacific  Islands (2024)</t>
+          <t>Early-Onset Cancer Incidence Disparities Between Black and White Individuals in the US, 2003-2022 (2026)</t>
         </is>
       </c>
       <c r="D24" s="13" t="inlineStr">
         <is>
-          <t>38996557</t>
+          <t>41989785</t>
         </is>
       </c>
       <c r="E24" s="13" t="inlineStr">
         <is>
-          <t>10.1016/j.canep.2024.102611</t>
+          <t>10.1001/jamanetworkopen.2026.7529</t>
         </is>
       </c>
       <c r="F24" s="14" t="inlineStr">
@@ -24415,7 +24415,7 @@
     <row r="25">
       <c r="A25" s="13" t="inlineStr">
         <is>
-          <t>998</t>
+          <t>1637</t>
         </is>
       </c>
       <c r="B25" s="13" t="inlineStr">
@@ -24425,17 +24425,17 @@
       </c>
       <c r="C25" s="14" t="inlineStr">
         <is>
-          <t>Cancer-related risk factors and incidence of major cancers by race, gender and region; analysis of the NIH-AARP diet and health study (2017)</t>
+          <t>Cancer Incidence in the Hispanic Community Health Study/Study of Latinos (HCHS/SOL)—The Onco-SOL Ancillary Study (2025)</t>
         </is>
       </c>
       <c r="D25" s="13" t="inlineStr">
         <is>
-          <t>28854891</t>
+          <t>39808161</t>
         </is>
       </c>
       <c r="E25" s="13" t="inlineStr">
         <is>
-          <t>10.1186/s12885-017-3557-1</t>
+          <t>10.1158/1055-9965.epi-24-1325</t>
         </is>
       </c>
       <c r="F25" s="14" t="inlineStr">
@@ -24450,7 +24450,7 @@
     <row r="26">
       <c r="A26" s="13" t="inlineStr">
         <is>
-          <t>1101</t>
+          <t>1800</t>
         </is>
       </c>
       <c r="B26" s="13" t="inlineStr">
@@ -24460,17 +24460,17 @@
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>Cancer incidence in the Somali population of Olmsted County: A Rochester epidemiology project study (2023)</t>
+          <t>Rural–Urban Cancer Incidence and Trends in the United States, 2000 to 2019 (2024)</t>
         </is>
       </c>
       <c r="D26" s="13" t="inlineStr">
         <is>
-          <t>37740603</t>
+          <t>38801414</t>
         </is>
       </c>
       <c r="E26" s="13" t="inlineStr">
         <is>
-          <t>10.1002/cam4.6558</t>
+          <t>10.1158/1055-9965.epi-24-0072</t>
         </is>
       </c>
       <c r="F26" s="14" t="inlineStr">
@@ -24485,32 +24485,28 @@
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
         <is>
-          <t>1398</t>
+          <t>2163</t>
         </is>
       </c>
       <c r="B27" s="13" t="inlineStr">
         <is>
-          <t>INCLUDED (narrative)</t>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
         </is>
       </c>
       <c r="C27" s="14" t="inlineStr">
         <is>
-          <t>Early-Onset Cancer Incidence Disparities Between Black and White Individuals in the US, 2003-2022 (2026)</t>
-        </is>
-      </c>
-      <c r="D27" s="13" t="inlineStr">
-        <is>
-          <t>41989785</t>
-        </is>
-      </c>
+          <t>Estrogen receptor negative breast cancer incidence rates are similar in Ghanaian and Non-Hispanic Black women in the USA (2022)</t>
+        </is>
+      </c>
+      <c r="D27" s="13" t="inlineStr"/>
       <c r="E27" s="13" t="inlineStr">
         <is>
-          <t>10.1001/jamanetworkopen.2026.7529</t>
+          <t>10.1101/2022.02.21.22271266</t>
         </is>
       </c>
       <c r="F27" s="14" t="inlineStr">
         <is>
-          <t>LOW — narrative only</t>
+          <t>LOW — metadata-defensible</t>
         </is>
       </c>
       <c r="G27" s="15" t="inlineStr"/>
@@ -24520,142 +24516,41 @@
     <row r="28">
       <c r="A28" s="13" t="inlineStr">
         <is>
-          <t>1637</t>
+          <t>3713</t>
         </is>
       </c>
       <c r="B28" s="13" t="inlineStr">
         <is>
-          <t>INCLUDED (narrative)</t>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
         </is>
       </c>
       <c r="C28" s="14" t="inlineStr">
         <is>
-          <t>Cancer Incidence in the Hispanic Community Health Study/Study of Latinos (HCHS/SOL)—The Onco-SOL Ancillary Study (2025)</t>
-        </is>
-      </c>
-      <c r="D28" s="13" t="inlineStr">
-        <is>
-          <t>39808161</t>
-        </is>
-      </c>
+          <t>Cancer incidence and mortality among Filipinos in the USA and the Philippines: Patterns and trends (2016)</t>
+        </is>
+      </c>
+      <c r="D28" s="13" t="inlineStr"/>
       <c r="E28" s="13" t="inlineStr">
         <is>
-          <t>10.1158/1055-9965.epi-24-1325</t>
+          <t>10.1007/978-3-319-41118-7_3</t>
         </is>
       </c>
       <c r="F28" s="14" t="inlineStr">
         <is>
-          <t>LOW — narrative only</t>
+          <t>LOW — metadata-defensible</t>
         </is>
       </c>
       <c r="G28" s="15" t="inlineStr"/>
       <c r="H28" s="15" t="inlineStr"/>
       <c r="I28" s="16" t="inlineStr"/>
     </row>
-    <row r="29">
-      <c r="A29" s="13" t="inlineStr">
-        <is>
-          <t>1800</t>
-        </is>
-      </c>
-      <c r="B29" s="13" t="inlineStr">
-        <is>
-          <t>INCLUDED (narrative)</t>
-        </is>
-      </c>
-      <c r="C29" s="14" t="inlineStr">
-        <is>
-          <t>Rural–Urban Cancer Incidence and Trends in the United States, 2000 to 2019 (2024)</t>
-        </is>
-      </c>
-      <c r="D29" s="13" t="inlineStr">
-        <is>
-          <t>38801414</t>
-        </is>
-      </c>
-      <c r="E29" s="13" t="inlineStr">
-        <is>
-          <t>10.1158/1055-9965.epi-24-0072</t>
-        </is>
-      </c>
-      <c r="F29" s="14" t="inlineStr">
-        <is>
-          <t>LOW — narrative only</t>
-        </is>
-      </c>
-      <c r="G29" s="15" t="inlineStr"/>
-      <c r="H29" s="15" t="inlineStr"/>
-      <c r="I29" s="16" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="13" t="inlineStr">
-        <is>
-          <t>2163</t>
-        </is>
-      </c>
-      <c r="B30" s="13" t="inlineStr">
-        <is>
-          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
-        </is>
-      </c>
-      <c r="C30" s="14" t="inlineStr">
-        <is>
-          <t>Estrogen receptor negative breast cancer incidence rates are similar in Ghanaian and Non-Hispanic Black women in the USA (2022)</t>
-        </is>
-      </c>
-      <c r="D30" s="13" t="inlineStr"/>
-      <c r="E30" s="13" t="inlineStr">
-        <is>
-          <t>10.1101/2022.02.21.22271266</t>
-        </is>
-      </c>
-      <c r="F30" s="14" t="inlineStr">
-        <is>
-          <t>LOW — metadata-defensible</t>
-        </is>
-      </c>
-      <c r="G30" s="15" t="inlineStr"/>
-      <c r="H30" s="15" t="inlineStr"/>
-      <c r="I30" s="16" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="13" t="inlineStr">
-        <is>
-          <t>3713</t>
-        </is>
-      </c>
-      <c r="B31" s="13" t="inlineStr">
-        <is>
-          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
-        </is>
-      </c>
-      <c r="C31" s="14" t="inlineStr">
-        <is>
-          <t>Cancer incidence and mortality among Filipinos in the USA and the Philippines: Patterns and trends (2016)</t>
-        </is>
-      </c>
-      <c r="D31" s="13" t="inlineStr"/>
-      <c r="E31" s="13" t="inlineStr">
-        <is>
-          <t>10.1007/978-3-319-41118-7_3</t>
-        </is>
-      </c>
-      <c r="F31" s="14" t="inlineStr">
-        <is>
-          <t>LOW — metadata-defensible</t>
-        </is>
-      </c>
-      <c r="G31" s="15" t="inlineStr"/>
-      <c r="H31" s="15" t="inlineStr"/>
-      <c r="I31" s="16" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I31"/>
+  <autoFilter ref="A1:I28"/>
   <dataValidations count="2">
-    <dataValidation sqref="G3:G31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G3:G28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="H3:H31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H3:H28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Include,Exclude"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Classify rec 426 (Quinn 2025, invasive lobular carcinoma trends) — kept narrative on scope
rec 426 does report all-age NHW-comparable ILC rates (NHW 13.52, NHB 8.60,
Hispanic 7.52 per 100k; IRRs 0.64 / 0.56), so it is data-eligible, but ILC is
a histologic subtype outside the review's receptor-defined molecular-subtype
cell set (HR/HER2/TNBC). Author decision this session: keep the subtype axis
receptor-defined; summarize ILC narratively. Extractable values recorded in
outputs/Reclassification_log.md for transparency. Workbook Sheet 6 now 25.
78 cells, headline results, and crosschecks A-F unchanged.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CuLT4FKRBtsU22Vwfjj2qn
</commit_message>
<xml_diff>
--- a/meta_agents/search_v2/outputs/Author_Validation_Workbook.xlsx
+++ b/meta_agents/search_v2/outputs/Author_Validation_Workbook.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'2_TA_Excluded_Sample'!$A$1:$E$152</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'3_Extraction_Verification'!$A$1:$M$147</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'4_RoB_Review'!$A$1:$Q$45</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'6_FullText_ToObtain'!$A$1:$I$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'6_FullText_ToObtain'!$A$1:$I$27</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -23574,7 +23574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -24100,7 +24100,7 @@
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
         <is>
-          <t>426</t>
+          <t>510</t>
         </is>
       </c>
       <c r="B16" s="13" t="inlineStr">
@@ -24110,17 +24110,17 @@
       </c>
       <c r="C16" s="14" t="inlineStr">
         <is>
-          <t>Trends in Incidence of Invasive Lobular Carcinoma of the Breast by Race: Patterns by Age, Cancer Stage, and Socioeconomic Factors in the United States, 1992-2019 (2025)</t>
+          <t>Cancer statistics for Asian Americans, Native Hawaiians, and Pacific Islanders, 2016: Converging incidence in males and females (2016)</t>
         </is>
       </c>
       <c r="D16" s="13" t="inlineStr">
         <is>
-          <t>39837694</t>
+          <t>26766789</t>
         </is>
       </c>
       <c r="E16" s="13" t="inlineStr">
         <is>
-          <t>10.1016/j.clbc.2024.12.015</t>
+          <t>10.3322/caac.21335</t>
         </is>
       </c>
       <c r="F16" s="14" t="inlineStr">
@@ -24135,7 +24135,7 @@
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>510</t>
+          <t>516</t>
         </is>
       </c>
       <c r="B17" s="13" t="inlineStr">
@@ -24145,17 +24145,17 @@
       </c>
       <c r="C17" s="14" t="inlineStr">
         <is>
-          <t>Cancer statistics for Asian Americans, Native Hawaiians, and Pacific Islanders, 2016: Converging incidence in males and females (2016)</t>
+          <t>The role of area-level socioeconomic disadvantage in racial disparities in cancer incidence in metropolitan Detroit (2023)</t>
         </is>
       </c>
       <c r="D17" s="13" t="inlineStr">
         <is>
-          <t>26766789</t>
+          <t>37184135</t>
         </is>
       </c>
       <c r="E17" s="13" t="inlineStr">
         <is>
-          <t>10.3322/caac.21335</t>
+          <t>10.1002/cam4.6065</t>
         </is>
       </c>
       <c r="F17" s="14" t="inlineStr">
@@ -24170,7 +24170,7 @@
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
         <is>
-          <t>516</t>
+          <t>565</t>
         </is>
       </c>
       <c r="B18" s="13" t="inlineStr">
@@ -24180,17 +24180,17 @@
       </c>
       <c r="C18" s="14" t="inlineStr">
         <is>
-          <t>The role of area-level socioeconomic disadvantage in racial disparities in cancer incidence in metropolitan Detroit (2023)</t>
+          <t>Cancer in Guam and Hawaii: A comparison of two U.S. Island populations (2017)</t>
         </is>
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>37184135</t>
+          <t>29120826</t>
         </is>
       </c>
       <c r="E18" s="13" t="inlineStr">
         <is>
-          <t>10.1002/cam4.6065</t>
+          <t>10.1016/j.canep.2017.08.005</t>
         </is>
       </c>
       <c r="F18" s="14" t="inlineStr">
@@ -24205,7 +24205,7 @@
     <row r="19">
       <c r="A19" s="13" t="inlineStr">
         <is>
-          <t>565</t>
+          <t>751</t>
         </is>
       </c>
       <c r="B19" s="13" t="inlineStr">
@@ -24215,17 +24215,17 @@
       </c>
       <c r="C19" s="14" t="inlineStr">
         <is>
-          <t>Cancer in Guam and Hawaii: A comparison of two U.S. Island populations (2017)</t>
+          <t>Population-based statistics for women diagnosed with inflammatory breast cancer (United States) (2004)</t>
         </is>
       </c>
       <c r="D19" s="13" t="inlineStr">
         <is>
-          <t>29120826</t>
+          <t>15090727</t>
         </is>
       </c>
       <c r="E19" s="13" t="inlineStr">
         <is>
-          <t>10.1016/j.canep.2017.08.005</t>
+          <t>10.1023/b:caco.0000024222.61114.18</t>
         </is>
       </c>
       <c r="F19" s="14" t="inlineStr">
@@ -24240,7 +24240,7 @@
     <row r="20">
       <c r="A20" s="13" t="inlineStr">
         <is>
-          <t>751</t>
+          <t>754</t>
         </is>
       </c>
       <c r="B20" s="13" t="inlineStr">
@@ -24250,17 +24250,17 @@
       </c>
       <c r="C20" s="14" t="inlineStr">
         <is>
-          <t>Population-based statistics for women diagnosed with inflammatory breast cancer (United States) (2004)</t>
+          <t>Breast cancer incidence and stage at diagnosis in the six US-Affiliated Pacific  Islands (2024)</t>
         </is>
       </c>
       <c r="D20" s="13" t="inlineStr">
         <is>
-          <t>15090727</t>
+          <t>38996557</t>
         </is>
       </c>
       <c r="E20" s="13" t="inlineStr">
         <is>
-          <t>10.1023/b:caco.0000024222.61114.18</t>
+          <t>10.1016/j.canep.2024.102611</t>
         </is>
       </c>
       <c r="F20" s="14" t="inlineStr">
@@ -24275,7 +24275,7 @@
     <row r="21">
       <c r="A21" s="13" t="inlineStr">
         <is>
-          <t>754</t>
+          <t>998</t>
         </is>
       </c>
       <c r="B21" s="13" t="inlineStr">
@@ -24285,17 +24285,17 @@
       </c>
       <c r="C21" s="14" t="inlineStr">
         <is>
-          <t>Breast cancer incidence and stage at diagnosis in the six US-Affiliated Pacific  Islands (2024)</t>
+          <t>Cancer-related risk factors and incidence of major cancers by race, gender and region; analysis of the NIH-AARP diet and health study (2017)</t>
         </is>
       </c>
       <c r="D21" s="13" t="inlineStr">
         <is>
-          <t>38996557</t>
+          <t>28854891</t>
         </is>
       </c>
       <c r="E21" s="13" t="inlineStr">
         <is>
-          <t>10.1016/j.canep.2024.102611</t>
+          <t>10.1186/s12885-017-3557-1</t>
         </is>
       </c>
       <c r="F21" s="14" t="inlineStr">
@@ -24310,7 +24310,7 @@
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
         <is>
-          <t>998</t>
+          <t>1101</t>
         </is>
       </c>
       <c r="B22" s="13" t="inlineStr">
@@ -24320,17 +24320,17 @@
       </c>
       <c r="C22" s="14" t="inlineStr">
         <is>
-          <t>Cancer-related risk factors and incidence of major cancers by race, gender and region; analysis of the NIH-AARP diet and health study (2017)</t>
+          <t>Cancer incidence in the Somali population of Olmsted County: A Rochester epidemiology project study (2023)</t>
         </is>
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
-          <t>28854891</t>
+          <t>37740603</t>
         </is>
       </c>
       <c r="E22" s="13" t="inlineStr">
         <is>
-          <t>10.1186/s12885-017-3557-1</t>
+          <t>10.1002/cam4.6558</t>
         </is>
       </c>
       <c r="F22" s="14" t="inlineStr">
@@ -24345,7 +24345,7 @@
     <row r="23">
       <c r="A23" s="13" t="inlineStr">
         <is>
-          <t>1101</t>
+          <t>1398</t>
         </is>
       </c>
       <c r="B23" s="13" t="inlineStr">
@@ -24355,17 +24355,17 @@
       </c>
       <c r="C23" s="14" t="inlineStr">
         <is>
-          <t>Cancer incidence in the Somali population of Olmsted County: A Rochester epidemiology project study (2023)</t>
+          <t>Early-Onset Cancer Incidence Disparities Between Black and White Individuals in the US, 2003-2022 (2026)</t>
         </is>
       </c>
       <c r="D23" s="13" t="inlineStr">
         <is>
-          <t>37740603</t>
+          <t>41989785</t>
         </is>
       </c>
       <c r="E23" s="13" t="inlineStr">
         <is>
-          <t>10.1002/cam4.6558</t>
+          <t>10.1001/jamanetworkopen.2026.7529</t>
         </is>
       </c>
       <c r="F23" s="14" t="inlineStr">
@@ -24380,7 +24380,7 @@
     <row r="24">
       <c r="A24" s="13" t="inlineStr">
         <is>
-          <t>1398</t>
+          <t>1637</t>
         </is>
       </c>
       <c r="B24" s="13" t="inlineStr">
@@ -24390,17 +24390,17 @@
       </c>
       <c r="C24" s="14" t="inlineStr">
         <is>
-          <t>Early-Onset Cancer Incidence Disparities Between Black and White Individuals in the US, 2003-2022 (2026)</t>
+          <t>Cancer Incidence in the Hispanic Community Health Study/Study of Latinos (HCHS/SOL)—The Onco-SOL Ancillary Study (2025)</t>
         </is>
       </c>
       <c r="D24" s="13" t="inlineStr">
         <is>
-          <t>41989785</t>
+          <t>39808161</t>
         </is>
       </c>
       <c r="E24" s="13" t="inlineStr">
         <is>
-          <t>10.1001/jamanetworkopen.2026.7529</t>
+          <t>10.1158/1055-9965.epi-24-1325</t>
         </is>
       </c>
       <c r="F24" s="14" t="inlineStr">
@@ -24415,7 +24415,7 @@
     <row r="25">
       <c r="A25" s="13" t="inlineStr">
         <is>
-          <t>1637</t>
+          <t>1800</t>
         </is>
       </c>
       <c r="B25" s="13" t="inlineStr">
@@ -24425,17 +24425,17 @@
       </c>
       <c r="C25" s="14" t="inlineStr">
         <is>
-          <t>Cancer Incidence in the Hispanic Community Health Study/Study of Latinos (HCHS/SOL)—The Onco-SOL Ancillary Study (2025)</t>
+          <t>Rural–Urban Cancer Incidence and Trends in the United States, 2000 to 2019 (2024)</t>
         </is>
       </c>
       <c r="D25" s="13" t="inlineStr">
         <is>
-          <t>39808161</t>
+          <t>38801414</t>
         </is>
       </c>
       <c r="E25" s="13" t="inlineStr">
         <is>
-          <t>10.1158/1055-9965.epi-24-1325</t>
+          <t>10.1158/1055-9965.epi-24-0072</t>
         </is>
       </c>
       <c r="F25" s="14" t="inlineStr">
@@ -24450,32 +24450,28 @@
     <row r="26">
       <c r="A26" s="13" t="inlineStr">
         <is>
-          <t>1800</t>
+          <t>2163</t>
         </is>
       </c>
       <c r="B26" s="13" t="inlineStr">
         <is>
-          <t>INCLUDED (narrative)</t>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
         </is>
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>Rural–Urban Cancer Incidence and Trends in the United States, 2000 to 2019 (2024)</t>
-        </is>
-      </c>
-      <c r="D26" s="13" t="inlineStr">
-        <is>
-          <t>38801414</t>
-        </is>
-      </c>
+          <t>Estrogen receptor negative breast cancer incidence rates are similar in Ghanaian and Non-Hispanic Black women in the USA (2022)</t>
+        </is>
+      </c>
+      <c r="D26" s="13" t="inlineStr"/>
       <c r="E26" s="13" t="inlineStr">
         <is>
-          <t>10.1158/1055-9965.epi-24-0072</t>
+          <t>10.1101/2022.02.21.22271266</t>
         </is>
       </c>
       <c r="F26" s="14" t="inlineStr">
         <is>
-          <t>LOW — narrative only</t>
+          <t>LOW — metadata-defensible</t>
         </is>
       </c>
       <c r="G26" s="15" t="inlineStr"/>
@@ -24485,7 +24481,7 @@
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
         <is>
-          <t>2163</t>
+          <t>3713</t>
         </is>
       </c>
       <c r="B27" s="13" t="inlineStr">
@@ -24495,13 +24491,13 @@
       </c>
       <c r="C27" s="14" t="inlineStr">
         <is>
-          <t>Estrogen receptor negative breast cancer incidence rates are similar in Ghanaian and Non-Hispanic Black women in the USA (2022)</t>
+          <t>Cancer incidence and mortality among Filipinos in the USA and the Philippines: Patterns and trends (2016)</t>
         </is>
       </c>
       <c r="D27" s="13" t="inlineStr"/>
       <c r="E27" s="13" t="inlineStr">
         <is>
-          <t>10.1101/2022.02.21.22271266</t>
+          <t>10.1007/978-3-319-41118-7_3</t>
         </is>
       </c>
       <c r="F27" s="14" t="inlineStr">
@@ -24513,44 +24509,13 @@
       <c r="H27" s="15" t="inlineStr"/>
       <c r="I27" s="16" t="inlineStr"/>
     </row>
-    <row r="28">
-      <c r="A28" s="13" t="inlineStr">
-        <is>
-          <t>3713</t>
-        </is>
-      </c>
-      <c r="B28" s="13" t="inlineStr">
-        <is>
-          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
-        </is>
-      </c>
-      <c r="C28" s="14" t="inlineStr">
-        <is>
-          <t>Cancer incidence and mortality among Filipinos in the USA and the Philippines: Patterns and trends (2016)</t>
-        </is>
-      </c>
-      <c r="D28" s="13" t="inlineStr"/>
-      <c r="E28" s="13" t="inlineStr">
-        <is>
-          <t>10.1007/978-3-319-41118-7_3</t>
-        </is>
-      </c>
-      <c r="F28" s="14" t="inlineStr">
-        <is>
-          <t>LOW — metadata-defensible</t>
-        </is>
-      </c>
-      <c r="G28" s="15" t="inlineStr"/>
-      <c r="H28" s="15" t="inlineStr"/>
-      <c r="I28" s="16" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I28"/>
+  <autoFilter ref="A1:I27"/>
   <dataValidations count="2">
-    <dataValidation sqref="G3:G28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G3:G27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="H3:H28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H3:H27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Include,Exclude"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Classify 5 author-supplied PDFs (510/516/565/751/754) - all narrative, no upgrade
510 Torre 2016 (ACS AANHPI stats; breast = aggregate trend, subgroup tables are
all-sites/lung not breast; overlaps SEER subgroup reps).
516 Purrington 2023 (metro-Detroit breast IRRs NHB 0.96 / elevated TNBC, but
regional overlap of USCS-national reps; ADI focus).
565 Hernandez 2017 (Guam vs Hawaii island comparison; no NHW comparator).
754 Gopalani 2024 (six US-Affiliated Pacific Islands; no NHW comparator).
751 Wingo 2004 (inflammatory breast cancer; Black 1.6 vs White ~1.3, but IBC is a
niche subtype outside the receptor-defined cell set - same scope basis as rec 259/426).

Reasons in outputs/Reclassification_log.md; workbook Sheet 6 (to-obtain) now 20.
78 cells, headline results, and crosschecks A-F unchanged.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CuLT4FKRBtsU22Vwfjj2qn
</commit_message>
<xml_diff>
--- a/meta_agents/search_v2/outputs/Author_Validation_Workbook.xlsx
+++ b/meta_agents/search_v2/outputs/Author_Validation_Workbook.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'2_TA_Excluded_Sample'!$A$1:$E$152</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'3_Extraction_Verification'!$A$1:$M$147</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'4_RoB_Review'!$A$1:$Q$45</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'6_FullText_ToObtain'!$A$1:$I$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'6_FullText_ToObtain'!$A$1:$I$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -23574,7 +23574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -24100,7 +24100,7 @@
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
         <is>
-          <t>510</t>
+          <t>998</t>
         </is>
       </c>
       <c r="B16" s="13" t="inlineStr">
@@ -24110,17 +24110,17 @@
       </c>
       <c r="C16" s="14" t="inlineStr">
         <is>
-          <t>Cancer statistics for Asian Americans, Native Hawaiians, and Pacific Islanders, 2016: Converging incidence in males and females (2016)</t>
+          <t>Cancer-related risk factors and incidence of major cancers by race, gender and region; analysis of the NIH-AARP diet and health study (2017)</t>
         </is>
       </c>
       <c r="D16" s="13" t="inlineStr">
         <is>
-          <t>26766789</t>
+          <t>28854891</t>
         </is>
       </c>
       <c r="E16" s="13" t="inlineStr">
         <is>
-          <t>10.3322/caac.21335</t>
+          <t>10.1186/s12885-017-3557-1</t>
         </is>
       </c>
       <c r="F16" s="14" t="inlineStr">
@@ -24135,7 +24135,7 @@
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>516</t>
+          <t>1101</t>
         </is>
       </c>
       <c r="B17" s="13" t="inlineStr">
@@ -24145,17 +24145,17 @@
       </c>
       <c r="C17" s="14" t="inlineStr">
         <is>
-          <t>The role of area-level socioeconomic disadvantage in racial disparities in cancer incidence in metropolitan Detroit (2023)</t>
+          <t>Cancer incidence in the Somali population of Olmsted County: A Rochester epidemiology project study (2023)</t>
         </is>
       </c>
       <c r="D17" s="13" t="inlineStr">
         <is>
-          <t>37184135</t>
+          <t>37740603</t>
         </is>
       </c>
       <c r="E17" s="13" t="inlineStr">
         <is>
-          <t>10.1002/cam4.6065</t>
+          <t>10.1002/cam4.6558</t>
         </is>
       </c>
       <c r="F17" s="14" t="inlineStr">
@@ -24170,7 +24170,7 @@
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
         <is>
-          <t>565</t>
+          <t>1398</t>
         </is>
       </c>
       <c r="B18" s="13" t="inlineStr">
@@ -24180,17 +24180,17 @@
       </c>
       <c r="C18" s="14" t="inlineStr">
         <is>
-          <t>Cancer in Guam and Hawaii: A comparison of two U.S. Island populations (2017)</t>
+          <t>Early-Onset Cancer Incidence Disparities Between Black and White Individuals in the US, 2003-2022 (2026)</t>
         </is>
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>29120826</t>
+          <t>41989785</t>
         </is>
       </c>
       <c r="E18" s="13" t="inlineStr">
         <is>
-          <t>10.1016/j.canep.2017.08.005</t>
+          <t>10.1001/jamanetworkopen.2026.7529</t>
         </is>
       </c>
       <c r="F18" s="14" t="inlineStr">
@@ -24205,7 +24205,7 @@
     <row r="19">
       <c r="A19" s="13" t="inlineStr">
         <is>
-          <t>751</t>
+          <t>1637</t>
         </is>
       </c>
       <c r="B19" s="13" t="inlineStr">
@@ -24215,17 +24215,17 @@
       </c>
       <c r="C19" s="14" t="inlineStr">
         <is>
-          <t>Population-based statistics for women diagnosed with inflammatory breast cancer (United States) (2004)</t>
+          <t>Cancer Incidence in the Hispanic Community Health Study/Study of Latinos (HCHS/SOL)—The Onco-SOL Ancillary Study (2025)</t>
         </is>
       </c>
       <c r="D19" s="13" t="inlineStr">
         <is>
-          <t>15090727</t>
+          <t>39808161</t>
         </is>
       </c>
       <c r="E19" s="13" t="inlineStr">
         <is>
-          <t>10.1023/b:caco.0000024222.61114.18</t>
+          <t>10.1158/1055-9965.epi-24-1325</t>
         </is>
       </c>
       <c r="F19" s="14" t="inlineStr">
@@ -24240,7 +24240,7 @@
     <row r="20">
       <c r="A20" s="13" t="inlineStr">
         <is>
-          <t>754</t>
+          <t>1800</t>
         </is>
       </c>
       <c r="B20" s="13" t="inlineStr">
@@ -24250,17 +24250,17 @@
       </c>
       <c r="C20" s="14" t="inlineStr">
         <is>
-          <t>Breast cancer incidence and stage at diagnosis in the six US-Affiliated Pacific  Islands (2024)</t>
+          <t>Rural–Urban Cancer Incidence and Trends in the United States, 2000 to 2019 (2024)</t>
         </is>
       </c>
       <c r="D20" s="13" t="inlineStr">
         <is>
-          <t>38996557</t>
+          <t>38801414</t>
         </is>
       </c>
       <c r="E20" s="13" t="inlineStr">
         <is>
-          <t>10.1016/j.canep.2024.102611</t>
+          <t>10.1158/1055-9965.epi-24-0072</t>
         </is>
       </c>
       <c r="F20" s="14" t="inlineStr">
@@ -24275,32 +24275,28 @@
     <row r="21">
       <c r="A21" s="13" t="inlineStr">
         <is>
-          <t>998</t>
+          <t>2163</t>
         </is>
       </c>
       <c r="B21" s="13" t="inlineStr">
         <is>
-          <t>INCLUDED (narrative)</t>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
         </is>
       </c>
       <c r="C21" s="14" t="inlineStr">
         <is>
-          <t>Cancer-related risk factors and incidence of major cancers by race, gender and region; analysis of the NIH-AARP diet and health study (2017)</t>
-        </is>
-      </c>
-      <c r="D21" s="13" t="inlineStr">
-        <is>
-          <t>28854891</t>
-        </is>
-      </c>
+          <t>Estrogen receptor negative breast cancer incidence rates are similar in Ghanaian and Non-Hispanic Black women in the USA (2022)</t>
+        </is>
+      </c>
+      <c r="D21" s="13" t="inlineStr"/>
       <c r="E21" s="13" t="inlineStr">
         <is>
-          <t>10.1186/s12885-017-3557-1</t>
+          <t>10.1101/2022.02.21.22271266</t>
         </is>
       </c>
       <c r="F21" s="14" t="inlineStr">
         <is>
-          <t>LOW — narrative only</t>
+          <t>LOW — metadata-defensible</t>
         </is>
       </c>
       <c r="G21" s="15" t="inlineStr"/>
@@ -24310,212 +24306,41 @@
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
         <is>
-          <t>1101</t>
+          <t>3713</t>
         </is>
       </c>
       <c r="B22" s="13" t="inlineStr">
         <is>
-          <t>INCLUDED (narrative)</t>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
         </is>
       </c>
       <c r="C22" s="14" t="inlineStr">
         <is>
-          <t>Cancer incidence in the Somali population of Olmsted County: A Rochester epidemiology project study (2023)</t>
-        </is>
-      </c>
-      <c r="D22" s="13" t="inlineStr">
-        <is>
-          <t>37740603</t>
-        </is>
-      </c>
+          <t>Cancer incidence and mortality among Filipinos in the USA and the Philippines: Patterns and trends (2016)</t>
+        </is>
+      </c>
+      <c r="D22" s="13" t="inlineStr"/>
       <c r="E22" s="13" t="inlineStr">
         <is>
-          <t>10.1002/cam4.6558</t>
+          <t>10.1007/978-3-319-41118-7_3</t>
         </is>
       </c>
       <c r="F22" s="14" t="inlineStr">
         <is>
-          <t>LOW — narrative only</t>
+          <t>LOW — metadata-defensible</t>
         </is>
       </c>
       <c r="G22" s="15" t="inlineStr"/>
       <c r="H22" s="15" t="inlineStr"/>
       <c r="I22" s="16" t="inlineStr"/>
     </row>
-    <row r="23">
-      <c r="A23" s="13" t="inlineStr">
-        <is>
-          <t>1398</t>
-        </is>
-      </c>
-      <c r="B23" s="13" t="inlineStr">
-        <is>
-          <t>INCLUDED (narrative)</t>
-        </is>
-      </c>
-      <c r="C23" s="14" t="inlineStr">
-        <is>
-          <t>Early-Onset Cancer Incidence Disparities Between Black and White Individuals in the US, 2003-2022 (2026)</t>
-        </is>
-      </c>
-      <c r="D23" s="13" t="inlineStr">
-        <is>
-          <t>41989785</t>
-        </is>
-      </c>
-      <c r="E23" s="13" t="inlineStr">
-        <is>
-          <t>10.1001/jamanetworkopen.2026.7529</t>
-        </is>
-      </c>
-      <c r="F23" s="14" t="inlineStr">
-        <is>
-          <t>LOW — narrative only</t>
-        </is>
-      </c>
-      <c r="G23" s="15" t="inlineStr"/>
-      <c r="H23" s="15" t="inlineStr"/>
-      <c r="I23" s="16" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="13" t="inlineStr">
-        <is>
-          <t>1637</t>
-        </is>
-      </c>
-      <c r="B24" s="13" t="inlineStr">
-        <is>
-          <t>INCLUDED (narrative)</t>
-        </is>
-      </c>
-      <c r="C24" s="14" t="inlineStr">
-        <is>
-          <t>Cancer Incidence in the Hispanic Community Health Study/Study of Latinos (HCHS/SOL)—The Onco-SOL Ancillary Study (2025)</t>
-        </is>
-      </c>
-      <c r="D24" s="13" t="inlineStr">
-        <is>
-          <t>39808161</t>
-        </is>
-      </c>
-      <c r="E24" s="13" t="inlineStr">
-        <is>
-          <t>10.1158/1055-9965.epi-24-1325</t>
-        </is>
-      </c>
-      <c r="F24" s="14" t="inlineStr">
-        <is>
-          <t>LOW — narrative only</t>
-        </is>
-      </c>
-      <c r="G24" s="15" t="inlineStr"/>
-      <c r="H24" s="15" t="inlineStr"/>
-      <c r="I24" s="16" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="13" t="inlineStr">
-        <is>
-          <t>1800</t>
-        </is>
-      </c>
-      <c r="B25" s="13" t="inlineStr">
-        <is>
-          <t>INCLUDED (narrative)</t>
-        </is>
-      </c>
-      <c r="C25" s="14" t="inlineStr">
-        <is>
-          <t>Rural–Urban Cancer Incidence and Trends in the United States, 2000 to 2019 (2024)</t>
-        </is>
-      </c>
-      <c r="D25" s="13" t="inlineStr">
-        <is>
-          <t>38801414</t>
-        </is>
-      </c>
-      <c r="E25" s="13" t="inlineStr">
-        <is>
-          <t>10.1158/1055-9965.epi-24-0072</t>
-        </is>
-      </c>
-      <c r="F25" s="14" t="inlineStr">
-        <is>
-          <t>LOW — narrative only</t>
-        </is>
-      </c>
-      <c r="G25" s="15" t="inlineStr"/>
-      <c r="H25" s="15" t="inlineStr"/>
-      <c r="I25" s="16" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="13" t="inlineStr">
-        <is>
-          <t>2163</t>
-        </is>
-      </c>
-      <c r="B26" s="13" t="inlineStr">
-        <is>
-          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
-        </is>
-      </c>
-      <c r="C26" s="14" t="inlineStr">
-        <is>
-          <t>Estrogen receptor negative breast cancer incidence rates are similar in Ghanaian and Non-Hispanic Black women in the USA (2022)</t>
-        </is>
-      </c>
-      <c r="D26" s="13" t="inlineStr"/>
-      <c r="E26" s="13" t="inlineStr">
-        <is>
-          <t>10.1101/2022.02.21.22271266</t>
-        </is>
-      </c>
-      <c r="F26" s="14" t="inlineStr">
-        <is>
-          <t>LOW — metadata-defensible</t>
-        </is>
-      </c>
-      <c r="G26" s="15" t="inlineStr"/>
-      <c r="H26" s="15" t="inlineStr"/>
-      <c r="I26" s="16" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="13" t="inlineStr">
-        <is>
-          <t>3713</t>
-        </is>
-      </c>
-      <c r="B27" s="13" t="inlineStr">
-        <is>
-          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
-        </is>
-      </c>
-      <c r="C27" s="14" t="inlineStr">
-        <is>
-          <t>Cancer incidence and mortality among Filipinos in the USA and the Philippines: Patterns and trends (2016)</t>
-        </is>
-      </c>
-      <c r="D27" s="13" t="inlineStr"/>
-      <c r="E27" s="13" t="inlineStr">
-        <is>
-          <t>10.1007/978-3-319-41118-7_3</t>
-        </is>
-      </c>
-      <c r="F27" s="14" t="inlineStr">
-        <is>
-          <t>LOW — metadata-defensible</t>
-        </is>
-      </c>
-      <c r="G27" s="15" t="inlineStr"/>
-      <c r="H27" s="15" t="inlineStr"/>
-      <c r="I27" s="16" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I27"/>
+  <autoFilter ref="A1:I22"/>
   <dataValidations count="2">
-    <dataValidation sqref="G3:G27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G3:G22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="H3:H27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H3:H22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Include,Exclude"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Classify 3 author-supplied PDFs (1398/1101/998) - all narrative, no upgrade
1398 Lawrence 2026 (early-onset Black-vs-White IRR trend; age-restricted).
1101 Mohamed 2023 (Somali-vs-non-Somali rate ratio, single county; Somali not a
review cell group, comparator not national NHW).
998 Akinyemiju 2017 (NIH-AARP risk-factor cohort; breast HRs by adherence, ages
50-71; cohort/HR metric, not a population-based race-vs-NHW incidence rate).

Reasons in outputs/Reclassification_log.md; workbook Sheet 6 (to-obtain) now 17.
78 cells, headline results, and crosschecks A-F unchanged.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CuLT4FKRBtsU22Vwfjj2qn
</commit_message>
<xml_diff>
--- a/meta_agents/search_v2/outputs/Author_Validation_Workbook.xlsx
+++ b/meta_agents/search_v2/outputs/Author_Validation_Workbook.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'2_TA_Excluded_Sample'!$A$1:$E$152</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'3_Extraction_Verification'!$A$1:$M$147</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'4_RoB_Review'!$A$1:$Q$45</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'6_FullText_ToObtain'!$A$1:$I$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'6_FullText_ToObtain'!$A$1:$I$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -23574,7 +23574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -24100,7 +24100,7 @@
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
         <is>
-          <t>998</t>
+          <t>1637</t>
         </is>
       </c>
       <c r="B16" s="13" t="inlineStr">
@@ -24110,17 +24110,17 @@
       </c>
       <c r="C16" s="14" t="inlineStr">
         <is>
-          <t>Cancer-related risk factors and incidence of major cancers by race, gender and region; analysis of the NIH-AARP diet and health study (2017)</t>
+          <t>Cancer Incidence in the Hispanic Community Health Study/Study of Latinos (HCHS/SOL)—The Onco-SOL Ancillary Study (2025)</t>
         </is>
       </c>
       <c r="D16" s="13" t="inlineStr">
         <is>
-          <t>28854891</t>
+          <t>39808161</t>
         </is>
       </c>
       <c r="E16" s="13" t="inlineStr">
         <is>
-          <t>10.1186/s12885-017-3557-1</t>
+          <t>10.1158/1055-9965.epi-24-1325</t>
         </is>
       </c>
       <c r="F16" s="14" t="inlineStr">
@@ -24135,7 +24135,7 @@
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>1101</t>
+          <t>1800</t>
         </is>
       </c>
       <c r="B17" s="13" t="inlineStr">
@@ -24145,17 +24145,17 @@
       </c>
       <c r="C17" s="14" t="inlineStr">
         <is>
-          <t>Cancer incidence in the Somali population of Olmsted County: A Rochester epidemiology project study (2023)</t>
+          <t>Rural–Urban Cancer Incidence and Trends in the United States, 2000 to 2019 (2024)</t>
         </is>
       </c>
       <c r="D17" s="13" t="inlineStr">
         <is>
-          <t>37740603</t>
+          <t>38801414</t>
         </is>
       </c>
       <c r="E17" s="13" t="inlineStr">
         <is>
-          <t>10.1002/cam4.6558</t>
+          <t>10.1158/1055-9965.epi-24-0072</t>
         </is>
       </c>
       <c r="F17" s="14" t="inlineStr">
@@ -24170,32 +24170,28 @@
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
         <is>
-          <t>1398</t>
+          <t>2163</t>
         </is>
       </c>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>INCLUDED (narrative)</t>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
         </is>
       </c>
       <c r="C18" s="14" t="inlineStr">
         <is>
-          <t>Early-Onset Cancer Incidence Disparities Between Black and White Individuals in the US, 2003-2022 (2026)</t>
-        </is>
-      </c>
-      <c r="D18" s="13" t="inlineStr">
-        <is>
-          <t>41989785</t>
-        </is>
-      </c>
+          <t>Estrogen receptor negative breast cancer incidence rates are similar in Ghanaian and Non-Hispanic Black women in the USA (2022)</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="inlineStr"/>
       <c r="E18" s="13" t="inlineStr">
         <is>
-          <t>10.1001/jamanetworkopen.2026.7529</t>
+          <t>10.1101/2022.02.21.22271266</t>
         </is>
       </c>
       <c r="F18" s="14" t="inlineStr">
         <is>
-          <t>LOW — narrative only</t>
+          <t>LOW — metadata-defensible</t>
         </is>
       </c>
       <c r="G18" s="15" t="inlineStr"/>
@@ -24205,142 +24201,41 @@
     <row r="19">
       <c r="A19" s="13" t="inlineStr">
         <is>
-          <t>1637</t>
+          <t>3713</t>
         </is>
       </c>
       <c r="B19" s="13" t="inlineStr">
         <is>
-          <t>INCLUDED (narrative)</t>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
         </is>
       </c>
       <c r="C19" s="14" t="inlineStr">
         <is>
-          <t>Cancer Incidence in the Hispanic Community Health Study/Study of Latinos (HCHS/SOL)—The Onco-SOL Ancillary Study (2025)</t>
-        </is>
-      </c>
-      <c r="D19" s="13" t="inlineStr">
-        <is>
-          <t>39808161</t>
-        </is>
-      </c>
+          <t>Cancer incidence and mortality among Filipinos in the USA and the Philippines: Patterns and trends (2016)</t>
+        </is>
+      </c>
+      <c r="D19" s="13" t="inlineStr"/>
       <c r="E19" s="13" t="inlineStr">
         <is>
-          <t>10.1158/1055-9965.epi-24-1325</t>
+          <t>10.1007/978-3-319-41118-7_3</t>
         </is>
       </c>
       <c r="F19" s="14" t="inlineStr">
         <is>
-          <t>LOW — narrative only</t>
+          <t>LOW — metadata-defensible</t>
         </is>
       </c>
       <c r="G19" s="15" t="inlineStr"/>
       <c r="H19" s="15" t="inlineStr"/>
       <c r="I19" s="16" t="inlineStr"/>
     </row>
-    <row r="20">
-      <c r="A20" s="13" t="inlineStr">
-        <is>
-          <t>1800</t>
-        </is>
-      </c>
-      <c r="B20" s="13" t="inlineStr">
-        <is>
-          <t>INCLUDED (narrative)</t>
-        </is>
-      </c>
-      <c r="C20" s="14" t="inlineStr">
-        <is>
-          <t>Rural–Urban Cancer Incidence and Trends in the United States, 2000 to 2019 (2024)</t>
-        </is>
-      </c>
-      <c r="D20" s="13" t="inlineStr">
-        <is>
-          <t>38801414</t>
-        </is>
-      </c>
-      <c r="E20" s="13" t="inlineStr">
-        <is>
-          <t>10.1158/1055-9965.epi-24-0072</t>
-        </is>
-      </c>
-      <c r="F20" s="14" t="inlineStr">
-        <is>
-          <t>LOW — narrative only</t>
-        </is>
-      </c>
-      <c r="G20" s="15" t="inlineStr"/>
-      <c r="H20" s="15" t="inlineStr"/>
-      <c r="I20" s="16" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="13" t="inlineStr">
-        <is>
-          <t>2163</t>
-        </is>
-      </c>
-      <c r="B21" s="13" t="inlineStr">
-        <is>
-          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
-        </is>
-      </c>
-      <c r="C21" s="14" t="inlineStr">
-        <is>
-          <t>Estrogen receptor negative breast cancer incidence rates are similar in Ghanaian and Non-Hispanic Black women in the USA (2022)</t>
-        </is>
-      </c>
-      <c r="D21" s="13" t="inlineStr"/>
-      <c r="E21" s="13" t="inlineStr">
-        <is>
-          <t>10.1101/2022.02.21.22271266</t>
-        </is>
-      </c>
-      <c r="F21" s="14" t="inlineStr">
-        <is>
-          <t>LOW — metadata-defensible</t>
-        </is>
-      </c>
-      <c r="G21" s="15" t="inlineStr"/>
-      <c r="H21" s="15" t="inlineStr"/>
-      <c r="I21" s="16" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="13" t="inlineStr">
-        <is>
-          <t>3713</t>
-        </is>
-      </c>
-      <c r="B22" s="13" t="inlineStr">
-        <is>
-          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
-        </is>
-      </c>
-      <c r="C22" s="14" t="inlineStr">
-        <is>
-          <t>Cancer incidence and mortality among Filipinos in the USA and the Philippines: Patterns and trends (2016)</t>
-        </is>
-      </c>
-      <c r="D22" s="13" t="inlineStr"/>
-      <c r="E22" s="13" t="inlineStr">
-        <is>
-          <t>10.1007/978-3-319-41118-7_3</t>
-        </is>
-      </c>
-      <c r="F22" s="14" t="inlineStr">
-        <is>
-          <t>LOW — metadata-defensible</t>
-        </is>
-      </c>
-      <c r="G22" s="15" t="inlineStr"/>
-      <c r="H22" s="15" t="inlineStr"/>
-      <c r="I22" s="16" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I22"/>
+  <autoFilter ref="A1:I19"/>
   <dataValidations count="2">
-    <dataValidation sqref="G3:G22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G3:G19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="H3:H22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H3:H19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Include,Exclude"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
rec 155 directly source-verified against Supplement 1 eTable 1 (national Total row)
Author supplied the full text and Supplement 1. eTable 1's Total (national) row
reports the between-group TNBC IRRs with CIs verbatim: Black 1.95 (1.93-1.98),
AI/AN 0.86 (0.80-0.93), Hispanic 0.86 (0.84-0.88), Asian/PI 0.70 (0.68-0.72) -
matching all four ledger representatives exactly (rates, IRRs, and CIs). This
confirms the directly-reported-IRR provenance (the national IRR/CI is reported
in the supplement, not merely computed). Ledger verification updated
abstract-verified -> source-verified-eTable1; supplement saved as 155_supp.pdf.
Workbook builder now treats a _supp PDF as obtaining its parent record, so the
verified rec 155 drops out of Sheet 6 (to-obtain now 16: 4 narrative + 12 excluded).
78 cells, headline results, and crosschecks A-F unchanged.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CuLT4FKRBtsU22Vwfjj2qn
</commit_message>
<xml_diff>
--- a/meta_agents/search_v2/outputs/Author_Validation_Workbook.xlsx
+++ b/meta_agents/search_v2/outputs/Author_Validation_Workbook.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'2_TA_Excluded_Sample'!$A$1:$E$152</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'3_Extraction_Verification'!$A$1:$M$147</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'4_RoB_Review'!$A$1:$Q$45</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'6_FullText_ToObtain'!$A$1:$I$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'6_FullText_ToObtain'!$A$1:$I$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -23574,7 +23574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -23677,32 +23677,32 @@
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>155</t>
+          <t>157</t>
         </is>
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>INCLUDED (quant-extracted)</t>
+          <t>EXCLUDED (Full text unavailable)</t>
         </is>
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
-          <t>State Variation in Racial and Ethnic Disparities in Incidence of Triple-Negative Breast Cancer among US Women (2023)</t>
+          <t>Breast cancer trends among black and white women in the United States (2005)</t>
         </is>
       </c>
       <c r="D3" s="13" t="inlineStr">
         <is>
-          <t>36862439</t>
+          <t>16258086</t>
         </is>
       </c>
       <c r="E3" s="13" t="inlineStr">
         <is>
-          <t>10.1001/jamaoncol.2022.7835</t>
+          <t>10.1200/jco.2004.01.0421</t>
         </is>
       </c>
       <c r="F3" s="14" t="inlineStr">
         <is>
-          <t>HIGH — extracted without main PDF</t>
+          <t>HIGH — not retrieved (possible missed study)</t>
         </is>
       </c>
       <c r="G3" s="15" t="inlineStr"/>
@@ -23712,7 +23712,7 @@
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
         <is>
-          <t>157</t>
+          <t>253</t>
         </is>
       </c>
       <c r="B4" s="13" t="inlineStr">
@@ -23722,19 +23722,15 @@
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>Breast cancer trends among black and white women in the United States (2005)</t>
+          <t>Breast cancer patterns and lifetime risk of developing breast cancer among Puerto Rican females. (2000)</t>
         </is>
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
-          <t>16258086</t>
-        </is>
-      </c>
-      <c r="E4" s="13" t="inlineStr">
-        <is>
-          <t>10.1200/jco.2004.01.0421</t>
-        </is>
-      </c>
+          <t>10761199</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="inlineStr"/>
       <c r="F4" s="14" t="inlineStr">
         <is>
           <t>HIGH — not retrieved (possible missed study)</t>
@@ -23747,7 +23743,7 @@
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>253</t>
+          <t>415</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
@@ -23757,12 +23753,12 @@
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>Breast cancer patterns and lifetime risk of developing breast cancer among Puerto Rican females. (2000)</t>
+          <t>Women's cancers among Alaska Natives 1969-2003. (2006)</t>
         </is>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>10761199</t>
+          <t>17929614</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr"/>
@@ -23778,7 +23774,7 @@
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
         <is>
-          <t>415</t>
+          <t>424</t>
         </is>
       </c>
       <c r="B6" s="13" t="inlineStr">
@@ -23788,12 +23784,12 @@
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>Women's cancers among Alaska Natives 1969-2003. (2006)</t>
+          <t>Breast cancer in a multiethnic cohort in Hawaii and Los Angeles: Risk factor-adjusted incidence in Japanese equals and in Hawaiians exceeds that in whites (2002)</t>
         </is>
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>17929614</t>
+          <t>12223421</t>
         </is>
       </c>
       <c r="E6" s="13" t="inlineStr"/>
@@ -23809,7 +23805,7 @@
     <row r="7">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t>424</t>
+          <t>428</t>
         </is>
       </c>
       <c r="B7" s="13" t="inlineStr">
@@ -23819,12 +23815,12 @@
       </c>
       <c r="C7" s="14" t="inlineStr">
         <is>
-          <t>Breast cancer in a multiethnic cohort in Hawaii and Los Angeles: Risk factor-adjusted incidence in Japanese equals and in Hawaiians exceeds that in whites (2002)</t>
+          <t>Women's cancers among Alaska Natives: [corrected] 1969-2003. (2007)</t>
         </is>
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>12223421</t>
+          <t>18323374</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr"/>
@@ -23840,7 +23836,7 @@
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
         <is>
-          <t>428</t>
+          <t>476</t>
         </is>
       </c>
       <c r="B8" s="13" t="inlineStr">
@@ -23850,15 +23846,19 @@
       </c>
       <c r="C8" s="14" t="inlineStr">
         <is>
-          <t>Women's cancers among Alaska Natives: [corrected] 1969-2003. (2007)</t>
+          <t>Rural–urban disparities in breast cancer incidence among US women aged 20–49: trends by race/ethnicity, stage, poverty, and state from 2000–2019 (2026)</t>
         </is>
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>18323374</t>
-        </is>
-      </c>
-      <c r="E8" s="13" t="inlineStr"/>
+          <t>41665696</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>10.1007/s10552-026-02134-3</t>
+        </is>
+      </c>
       <c r="F8" s="14" t="inlineStr">
         <is>
           <t>HIGH — not retrieved (possible missed study)</t>
@@ -23871,7 +23871,7 @@
     <row r="9">
       <c r="A9" s="13" t="inlineStr">
         <is>
-          <t>476</t>
+          <t>2038</t>
         </is>
       </c>
       <c r="B9" s="13" t="inlineStr">
@@ -23881,19 +23881,11 @@
       </c>
       <c r="C9" s="14" t="inlineStr">
         <is>
-          <t>Rural–urban disparities in breast cancer incidence among US women aged 20–49: trends by race/ethnicity, stage, poverty, and state from 2000–2019 (2026)</t>
-        </is>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
-        <is>
-          <t>41665696</t>
-        </is>
-      </c>
-      <c r="E9" s="13" t="inlineStr">
-        <is>
-          <t>10.1007/s10552-026-02134-3</t>
-        </is>
-      </c>
+          <t>Incidence trends in triple-negative breast cancer among women in the United States from 2010 to 2019 by race/ethnicity, age and tumor stage (2023)</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr"/>
+      <c r="E9" s="13" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr">
         <is>
           <t>HIGH — not retrieved (possible missed study)</t>
@@ -23906,7 +23898,7 @@
     <row r="10">
       <c r="A10" s="13" t="inlineStr">
         <is>
-          <t>2038</t>
+          <t>3116</t>
         </is>
       </c>
       <c r="B10" s="13" t="inlineStr">
@@ -23916,11 +23908,15 @@
       </c>
       <c r="C10" s="14" t="inlineStr">
         <is>
-          <t>Incidence trends in triple-negative breast cancer among women in the United States from 2010 to 2019 by race/ethnicity, age and tumor stage (2023)</t>
+          <t>Time trends and racial differences in female breast cancer incidence in Pennsylvania, 1985-2004 (2011)</t>
         </is>
       </c>
       <c r="D10" s="13" t="inlineStr"/>
-      <c r="E10" s="13" t="inlineStr"/>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>10.1089/jwh.2010.2082</t>
+        </is>
+      </c>
       <c r="F10" s="14" t="inlineStr">
         <is>
           <t>HIGH — not retrieved (possible missed study)</t>
@@ -23933,7 +23929,7 @@
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>3116</t>
+          <t>3268</t>
         </is>
       </c>
       <c r="B11" s="13" t="inlineStr">
@@ -23943,15 +23939,15 @@
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
-          <t>Time trends and racial differences in female breast cancer incidence in Pennsylvania, 1985-2004 (2011)</t>
-        </is>
-      </c>
-      <c r="D11" s="13" t="inlineStr"/>
-      <c r="E11" s="13" t="inlineStr">
-        <is>
-          <t>10.1089/jwh.2010.2082</t>
-        </is>
-      </c>
+          <t>Improving cancer incidence estimates for American Indians in Wisconsin (2007)</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>17844709</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr">
         <is>
           <t>HIGH — not retrieved (possible missed study)</t>
@@ -23964,28 +23960,32 @@
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>3268</t>
+          <t>251</t>
         </is>
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>EXCLUDED (Full text unavailable)</t>
+          <t>EXCLUDED (Did not report the outcome of interest)</t>
         </is>
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>Improving cancer incidence estimates for American Indians in Wisconsin (2007)</t>
+          <t>Triple-negative breast cancer incidence in the United States: ecological correlations with area-level sociodemographics, healthcare, and health behaviors (2021)</t>
         </is>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>17844709</t>
-        </is>
-      </c>
-      <c r="E12" s="13" t="inlineStr"/>
+          <t>32671723</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>10.1007/s12282-020-01132-w</t>
+        </is>
+      </c>
       <c r="F12" s="14" t="inlineStr">
         <is>
-          <t>HIGH — not retrieved (possible missed study)</t>
+          <t>MED — excluded without full text</t>
         </is>
       </c>
       <c r="G12" s="15" t="inlineStr"/>
@@ -23995,32 +23995,32 @@
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>251</t>
+          <t>80</t>
         </is>
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>EXCLUDED (Did not report the outcome of interest)</t>
+          <t>INCLUDED (narrative)</t>
         </is>
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>Triple-negative breast cancer incidence in the United States: ecological correlations with area-level sociodemographics, healthcare, and health behaviors (2021)</t>
+          <t>Breast, Colorectal, and Prostate Cancer Incidence among Filipino Americans by Generational Status in the Multiethnic Cohort Study (2024)</t>
         </is>
       </c>
       <c r="D13" s="13" t="inlineStr">
         <is>
-          <t>32671723</t>
+          <t>39132985</t>
         </is>
       </c>
       <c r="E13" s="13" t="inlineStr">
         <is>
-          <t>10.1007/s12282-020-01132-w</t>
+          <t>10.1158/1055-9965.epi-24-0647</t>
         </is>
       </c>
       <c r="F13" s="14" t="inlineStr">
         <is>
-          <t>MED — excluded without full text</t>
+          <t>LOW — narrative only</t>
         </is>
       </c>
       <c r="G13" s="15" t="inlineStr"/>
@@ -24030,7 +24030,7 @@
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>402</t>
         </is>
       </c>
       <c r="B14" s="13" t="inlineStr">
@@ -24040,17 +24040,17 @@
       </c>
       <c r="C14" s="14" t="inlineStr">
         <is>
-          <t>Breast, Colorectal, and Prostate Cancer Incidence among Filipino Americans by Generational Status in the Multiethnic Cohort Study (2024)</t>
+          <t>Disparities in Breast Cancer Incidence, Mortality, and Quality of Care among African American and European American Women in South Carolina (2016)</t>
         </is>
       </c>
       <c r="D14" s="13" t="inlineStr">
         <is>
-          <t>39132985</t>
+          <t>26741869</t>
         </is>
       </c>
       <c r="E14" s="13" t="inlineStr">
         <is>
-          <t>10.1158/1055-9965.epi-24-0647</t>
+          <t>10.14423/smj.0000000000000396</t>
         </is>
       </c>
       <c r="F14" s="14" t="inlineStr">
@@ -24065,7 +24065,7 @@
     <row r="15">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>402</t>
+          <t>1637</t>
         </is>
       </c>
       <c r="B15" s="13" t="inlineStr">
@@ -24075,17 +24075,17 @@
       </c>
       <c r="C15" s="14" t="inlineStr">
         <is>
-          <t>Disparities in Breast Cancer Incidence, Mortality, and Quality of Care among African American and European American Women in South Carolina (2016)</t>
+          <t>Cancer Incidence in the Hispanic Community Health Study/Study of Latinos (HCHS/SOL)—The Onco-SOL Ancillary Study (2025)</t>
         </is>
       </c>
       <c r="D15" s="13" t="inlineStr">
         <is>
-          <t>26741869</t>
+          <t>39808161</t>
         </is>
       </c>
       <c r="E15" s="13" t="inlineStr">
         <is>
-          <t>10.14423/smj.0000000000000396</t>
+          <t>10.1158/1055-9965.epi-24-1325</t>
         </is>
       </c>
       <c r="F15" s="14" t="inlineStr">
@@ -24100,7 +24100,7 @@
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
         <is>
-          <t>1637</t>
+          <t>1800</t>
         </is>
       </c>
       <c r="B16" s="13" t="inlineStr">
@@ -24110,17 +24110,17 @@
       </c>
       <c r="C16" s="14" t="inlineStr">
         <is>
-          <t>Cancer Incidence in the Hispanic Community Health Study/Study of Latinos (HCHS/SOL)—The Onco-SOL Ancillary Study (2025)</t>
+          <t>Rural–Urban Cancer Incidence and Trends in the United States, 2000 to 2019 (2024)</t>
         </is>
       </c>
       <c r="D16" s="13" t="inlineStr">
         <is>
-          <t>39808161</t>
+          <t>38801414</t>
         </is>
       </c>
       <c r="E16" s="13" t="inlineStr">
         <is>
-          <t>10.1158/1055-9965.epi-24-1325</t>
+          <t>10.1158/1055-9965.epi-24-0072</t>
         </is>
       </c>
       <c r="F16" s="14" t="inlineStr">
@@ -24135,32 +24135,28 @@
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>1800</t>
+          <t>2163</t>
         </is>
       </c>
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>INCLUDED (narrative)</t>
+          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
         </is>
       </c>
       <c r="C17" s="14" t="inlineStr">
         <is>
-          <t>Rural–Urban Cancer Incidence and Trends in the United States, 2000 to 2019 (2024)</t>
-        </is>
-      </c>
-      <c r="D17" s="13" t="inlineStr">
-        <is>
-          <t>38801414</t>
-        </is>
-      </c>
+          <t>Estrogen receptor negative breast cancer incidence rates are similar in Ghanaian and Non-Hispanic Black women in the USA (2022)</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="inlineStr"/>
       <c r="E17" s="13" t="inlineStr">
         <is>
-          <t>10.1158/1055-9965.epi-24-0072</t>
+          <t>10.1101/2022.02.21.22271266</t>
         </is>
       </c>
       <c r="F17" s="14" t="inlineStr">
         <is>
-          <t>LOW — narrative only</t>
+          <t>LOW — metadata-defensible</t>
         </is>
       </c>
       <c r="G17" s="15" t="inlineStr"/>
@@ -24170,7 +24166,7 @@
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
         <is>
-          <t>2163</t>
+          <t>3713</t>
         </is>
       </c>
       <c r="B18" s="13" t="inlineStr">
@@ -24180,13 +24176,13 @@
       </c>
       <c r="C18" s="14" t="inlineStr">
         <is>
-          <t>Estrogen receptor negative breast cancer incidence rates are similar in Ghanaian and Non-Hispanic Black women in the USA (2022)</t>
+          <t>Cancer incidence and mortality among Filipinos in the USA and the Philippines: Patterns and trends (2016)</t>
         </is>
       </c>
       <c r="D18" s="13" t="inlineStr"/>
       <c r="E18" s="13" t="inlineStr">
         <is>
-          <t>10.1101/2022.02.21.22271266</t>
+          <t>10.1007/978-3-319-41118-7_3</t>
         </is>
       </c>
       <c r="F18" s="14" t="inlineStr">
@@ -24198,44 +24194,13 @@
       <c r="H18" s="15" t="inlineStr"/>
       <c r="I18" s="16" t="inlineStr"/>
     </row>
-    <row r="19">
-      <c r="A19" s="13" t="inlineStr">
-        <is>
-          <t>3713</t>
-        </is>
-      </c>
-      <c r="B19" s="13" t="inlineStr">
-        <is>
-          <t>EXCLUDED (Overlapping or duplicate dataset)</t>
-        </is>
-      </c>
-      <c r="C19" s="14" t="inlineStr">
-        <is>
-          <t>Cancer incidence and mortality among Filipinos in the USA and the Philippines: Patterns and trends (2016)</t>
-        </is>
-      </c>
-      <c r="D19" s="13" t="inlineStr"/>
-      <c r="E19" s="13" t="inlineStr">
-        <is>
-          <t>10.1007/978-3-319-41118-7_3</t>
-        </is>
-      </c>
-      <c r="F19" s="14" t="inlineStr">
-        <is>
-          <t>LOW — metadata-defensible</t>
-        </is>
-      </c>
-      <c r="G19" s="15" t="inlineStr"/>
-      <c r="H19" s="15" t="inlineStr"/>
-      <c r="I19" s="16" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I19"/>
+  <autoFilter ref="A1:I18"/>
   <dataValidations count="2">
-    <dataValidation sqref="G3:G19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G3:G18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="H3:H19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H3:H18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Include,Exclude"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>